<commit_message>
docs(qa): expand live execution to 143 checks; found 1 real defect (consignment PCI gap on deployed build)
Deepened the live execution (create/lifecycle flows across modules): 143 checks now executed (web UI 21 + API
122) -> 138 PASS / 1 FAIL / 4 PARTIAL. The 1 FAIL is a real live defect: a consignment-site note ACCEPTS + stores
a raw card number (HTTP 201) — the consignment PCI guard (commit 327b6e9) is committed in-branch but not in the
deployed build; leads/CIS correctly reject the same input. Reduced 'not auto-tested' from 854 to 821. Gaps
unchanged at 128 (FAILED): 53 Acumatica, 38 not-built, 25 email, 3 push, 9 other.

Co-Authored-By: claude-flow <ruv@ruv.net>
</commit_message>
<xml_diff>
--- a/docs/test-plan/Pulse_CRM_Module_Execution_Report.xlsx
+++ b/docs/test-plan/Pulse_CRM_Module_Execution_Report.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'GAPS (FAILED)'!$A$4:$F$132</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Executed (live)'!$A$3:$E$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Executed (live)'!$A$3:$E$146</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -123,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -157,6 +157,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -597,7 +600,7 @@
         <v>64</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D5" s="5" t="n">
         <v>0</v>
@@ -606,7 +609,7 @@
         <v>1</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
@@ -624,7 +627,7 @@
         <v>61</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D6" s="5" t="n">
         <v>0</v>
@@ -633,7 +636,7 @@
         <v>6</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
@@ -651,7 +654,7 @@
         <v>58</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D7" s="5" t="n">
         <v>0</v>
@@ -660,7 +663,7 @@
         <v>5</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
@@ -705,16 +708,16 @@
         <v>68</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="D9" s="5" t="n">
-        <v>0</v>
+        <v>9</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="E9" s="7" t="n">
         <v>5</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
@@ -732,7 +735,7 @@
         <v>54</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D10" s="5" t="n">
         <v>0</v>
@@ -741,7 +744,7 @@
         <v>6</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
@@ -759,7 +762,7 @@
         <v>53</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D11" s="5" t="n">
         <v>0</v>
@@ -768,7 +771,7 @@
         <v>3</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
@@ -813,7 +816,7 @@
         <v>60</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D13" s="5" t="n">
         <v>0</v>
@@ -822,7 +825,7 @@
         <v>3</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
@@ -840,7 +843,7 @@
         <v>62</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D14" s="5" t="n">
         <v>0</v>
@@ -849,7 +852,7 @@
         <v>6</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
@@ -921,7 +924,7 @@
         <v>68</v>
       </c>
       <c r="C17" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D17" s="5" t="n">
         <v>0</v>
@@ -930,7 +933,7 @@
         <v>2</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
@@ -948,7 +951,7 @@
         <v>60</v>
       </c>
       <c r="C18" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D18" s="5" t="n">
         <v>0</v>
@@ -957,7 +960,7 @@
         <v>2</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
@@ -1002,7 +1005,7 @@
         <v>58</v>
       </c>
       <c r="C20" s="6" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D20" s="5" t="n">
         <v>0</v>
@@ -1011,7 +1014,7 @@
         <v>7</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
@@ -1083,16 +1086,16 @@
         <v>1047</v>
       </c>
       <c r="C23" s="8" t="n">
-        <v>96</v>
+        <v>138</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E23" s="8" t="n">
         <v>128</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>822</v>
+        <v>776</v>
       </c>
       <c r="G23" s="8" t="inlineStr"/>
     </row>
@@ -5272,7 +5275,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E100"/>
+  <dimension ref="A1:E146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5285,7 +5288,7 @@
     <row r="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
-          <t>Live-executed checks — Web UI (21) + API (76)</t>
+          <t>Live-executed checks — Web UI (21) + API (122)</t>
         </is>
       </c>
     </row>
@@ -5454,7 +5457,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>WEB-UI</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
@@ -5464,7 +5467,7 @@
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>Web page renders: /customers</t>
+          <t>ACC-TC-004</t>
         </is>
       </c>
       <c r="D9" s="13" t="inlineStr">
@@ -5474,7 +5477,7 @@
       </c>
       <c r="E9" s="10" t="inlineStr">
         <is>
-          <t>Rendered correctly; saw ["Account","Pulse"]</t>
+          <t>Create account</t>
         </is>
       </c>
     </row>
@@ -5486,12 +5489,12 @@
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>Admin, Master Data &amp; RBAC</t>
+          <t>Accounts &amp; Customers</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>ADM-TC-001</t>
+          <t>ACC-TC-005</t>
         </is>
       </c>
       <c r="D10" s="13" t="inlineStr">
@@ -5501,7 +5504,7 @@
       </c>
       <c r="E10" s="10" t="inlineStr">
         <is>
-          <t>Admin lists users</t>
+          <t>Account detail loads</t>
         </is>
       </c>
     </row>
@@ -5513,39 +5516,39 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>Admin, Master Data &amp; RBAC</t>
+          <t>Accounts &amp; Customers</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>ADM-TC-002a</t>
-        </is>
-      </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>PASS</t>
+          <t>ACC-TC-011</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="E11" s="10" t="inlineStr">
         <is>
-          <t>TERRITORY_MANAGER denied admin user list (default-deny)</t>
+          <t>SALES_BD_REP create-account access controlled (400)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>WEB-UI</t>
         </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>Admin, Master Data &amp; RBAC</t>
+          <t>Accounts &amp; Customers</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>ADM-TC-002b</t>
+          <t>Web page renders: /customers</t>
         </is>
       </c>
       <c r="D12" s="13" t="inlineStr">
@@ -5555,7 +5558,7 @@
       </c>
       <c r="E12" s="10" t="inlineStr">
         <is>
-          <t>FINANCE denied admin user list (default-deny)</t>
+          <t>Rendered correctly; saw ["Account","Pulse"]</t>
         </is>
       </c>
     </row>
@@ -5572,7 +5575,7 @@
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>ADM-TC-002c</t>
+          <t>ADM-TC-001</t>
         </is>
       </c>
       <c r="D13" s="13" t="inlineStr">
@@ -5582,7 +5585,7 @@
       </c>
       <c r="E13" s="10" t="inlineStr">
         <is>
-          <t>SALES_BD_REP denied admin user list (default-deny)</t>
+          <t>Admin lists users</t>
         </is>
       </c>
     </row>
@@ -5599,7 +5602,7 @@
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>ADM-TC-010</t>
+          <t>ADM-TC-002a</t>
         </is>
       </c>
       <c r="D14" s="13" t="inlineStr">
@@ -5609,7 +5612,7 @@
       </c>
       <c r="E14" s="10" t="inlineStr">
         <is>
-          <t>System health readable by admin</t>
+          <t>TERRITORY_MANAGER denied admin user list (default-deny)</t>
         </is>
       </c>
     </row>
@@ -5626,7 +5629,7 @@
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>ADM-TC-011</t>
+          <t>ADM-TC-002b</t>
         </is>
       </c>
       <c r="D15" s="13" t="inlineStr">
@@ -5636,7 +5639,7 @@
       </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>Admin activity/audit log readable</t>
+          <t>FINANCE denied admin user list (default-deny)</t>
         </is>
       </c>
     </row>
@@ -5653,7 +5656,7 @@
       </c>
       <c r="C16" s="10" t="inlineStr">
         <is>
-          <t>ADM-TC-012</t>
+          <t>ADM-TC-002c</t>
         </is>
       </c>
       <c r="D16" s="13" t="inlineStr">
@@ -5663,14 +5666,14 @@
       </c>
       <c r="E16" s="10" t="inlineStr">
         <is>
-          <t>Non-admin denied activity log</t>
+          <t>SALES_BD_REP denied admin user list (default-deny)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>WEB-UI</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B17" s="10" t="inlineStr">
@@ -5680,7 +5683,7 @@
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>Web page renders: /admin/users</t>
+          <t>ADM-TC-010</t>
         </is>
       </c>
       <c r="D17" s="13" t="inlineStr">
@@ -5690,14 +5693,14 @@
       </c>
       <c r="E17" s="10" t="inlineStr">
         <is>
-          <t>Rendered correctly; saw ["User","Pulse"]</t>
+          <t>System health readable by admin</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>WEB-UI</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
@@ -5707,7 +5710,7 @@
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>Web page renders: /admin/roles</t>
+          <t>ADM-TC-011</t>
         </is>
       </c>
       <c r="D18" s="13" t="inlineStr">
@@ -5717,14 +5720,14 @@
       </c>
       <c r="E18" s="10" t="inlineStr">
         <is>
-          <t>Rendered correctly; saw ["Role","Pulse"]</t>
+          <t>Admin activity/audit log readable</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>WEB-UI</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
@@ -5734,7 +5737,7 @@
       </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>Web page renders: /admin/integrations</t>
+          <t>ADM-TC-012</t>
         </is>
       </c>
       <c r="D19" s="13" t="inlineStr">
@@ -5744,7 +5747,7 @@
       </c>
       <c r="E19" s="10" t="inlineStr">
         <is>
-          <t>Rendered correctly; saw ["Integration","Pulse"]</t>
+          <t>Non-admin denied activity log</t>
         </is>
       </c>
     </row>
@@ -5756,12 +5759,12 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>Auth &amp; Session</t>
+          <t>Admin, Master Data &amp; RBAC</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>AUTH-TC-001</t>
+          <t>ADM-TC-020</t>
         </is>
       </c>
       <c r="D20" s="13" t="inlineStr">
@@ -5771,7 +5774,7 @@
       </c>
       <c r="E20" s="10" t="inlineStr">
         <is>
-          <t>Valid credentials returned a session + access token</t>
+          <t>Admin reset-password</t>
         </is>
       </c>
     </row>
@@ -5783,12 +5786,12 @@
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>Auth &amp; Session</t>
+          <t>Admin, Master Data &amp; RBAC</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>AUTH-TC-002</t>
+          <t>ADM-TC-021</t>
         </is>
       </c>
       <c r="D21" s="13" t="inlineStr">
@@ -5798,7 +5801,7 @@
       </c>
       <c r="E21" s="10" t="inlineStr">
         <is>
-          <t>Wrong password rejected</t>
+          <t>Admin update user</t>
         </is>
       </c>
     </row>
@@ -5810,12 +5813,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>Auth &amp; Session</t>
+          <t>Admin, Master Data &amp; RBAC</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>AUTH-TC-003</t>
+          <t>ADM-TC-022</t>
         </is>
       </c>
       <c r="D22" s="13" t="inlineStr">
@@ -5825,7 +5828,7 @@
       </c>
       <c r="E22" s="10" t="inlineStr">
         <is>
-          <t>Unknown email rejected</t>
+          <t>List roles</t>
         </is>
       </c>
     </row>
@@ -5837,12 +5840,12 @@
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>Auth &amp; Session</t>
+          <t>Admin, Master Data &amp; RBAC</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>AUTH-TC-004</t>
+          <t>ADM-TC-023</t>
         </is>
       </c>
       <c r="D23" s="13" t="inlineStr">
@@ -5852,24 +5855,24 @@
       </c>
       <c r="E23" s="10" t="inlineStr">
         <is>
-          <t>Protected endpoint requires auth</t>
+          <t>TM denied admin reset-password</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>WEB-UI</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>Auth &amp; Session</t>
+          <t>Admin, Master Data &amp; RBAC</t>
         </is>
       </c>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>AUTH-TC-005</t>
+          <t>Web page renders: /admin/users</t>
         </is>
       </c>
       <c r="D24" s="13" t="inlineStr">
@@ -5879,7 +5882,7 @@
       </c>
       <c r="E24" s="10" t="inlineStr">
         <is>
-          <t>Invalid/garbage token rejected</t>
+          <t>Rendered correctly; saw ["User","Pulse"]</t>
         </is>
       </c>
     </row>
@@ -5891,12 +5894,12 @@
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>Auth &amp; Session</t>
+          <t>Admin, Master Data &amp; RBAC</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>Login (web UI) as SUPER_ADMIN</t>
+          <t>Web page renders: /admin/roles</t>
         </is>
       </c>
       <c r="D25" s="13" t="inlineStr">
@@ -5906,24 +5909,24 @@
       </c>
       <c r="E25" s="10" t="inlineStr">
         <is>
-          <t>Logged in, redirected to app</t>
+          <t>Rendered correctly; saw ["Role","Pulse"]</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>WEB-UI</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>CIS &amp; Credit Onboarding</t>
+          <t>Admin, Master Data &amp; RBAC</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>CIS-TC-001</t>
+          <t>Web page renders: /admin/integrations</t>
         </is>
       </c>
       <c r="D26" s="13" t="inlineStr">
@@ -5933,7 +5936,7 @@
       </c>
       <c r="E26" s="10" t="inlineStr">
         <is>
-          <t>FINANCE can read CIS finance queue</t>
+          <t>Rendered correctly; saw ["Integration","Pulse"]</t>
         </is>
       </c>
     </row>
@@ -5945,12 +5948,12 @@
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>CIS &amp; Credit Onboarding</t>
+          <t>Auth &amp; Session</t>
         </is>
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>CIS-TC-002</t>
+          <t>AUTH-TC-001</t>
         </is>
       </c>
       <c r="D27" s="13" t="inlineStr">
@@ -5960,24 +5963,24 @@
       </c>
       <c r="E27" s="10" t="inlineStr">
         <is>
-          <t>TM denied CIS finance queue</t>
+          <t>Valid credentials returned a session + access token</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t>WEB-UI</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>Calendar</t>
+          <t>Auth &amp; Session</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>Web page renders: /calendar</t>
+          <t>AUTH-TC-002</t>
         </is>
       </c>
       <c r="D28" s="13" t="inlineStr">
@@ -5987,7 +5990,7 @@
       </c>
       <c r="E28" s="10" t="inlineStr">
         <is>
-          <t>Rendered correctly; saw ["Calendar","Pulse"]</t>
+          <t>Wrong password rejected</t>
         </is>
       </c>
     </row>
@@ -5999,12 +6002,12 @@
       </c>
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>Consignment</t>
+          <t>Auth &amp; Session</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>CON-TC-001</t>
+          <t>AUTH-TC-003</t>
         </is>
       </c>
       <c r="D29" s="13" t="inlineStr">
@@ -6014,7 +6017,7 @@
       </c>
       <c r="E29" s="10" t="inlineStr">
         <is>
-          <t>Consignment sites 200</t>
+          <t>Unknown email rejected</t>
         </is>
       </c>
     </row>
@@ -6026,12 +6029,12 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>Consignment</t>
+          <t>Auth &amp; Session</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>CON-TC-002</t>
+          <t>AUTH-TC-004</t>
         </is>
       </c>
       <c r="D30" s="13" t="inlineStr">
@@ -6041,7 +6044,7 @@
       </c>
       <c r="E30" s="10" t="inlineStr">
         <is>
-          <t>Consignment dashboard 200</t>
+          <t>Protected endpoint requires auth</t>
         </is>
       </c>
     </row>
@@ -6053,12 +6056,12 @@
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>Consignment</t>
+          <t>Auth &amp; Session</t>
         </is>
       </c>
       <c r="C31" s="10" t="inlineStr">
         <is>
-          <t>CON-TC-003</t>
+          <t>AUTH-TC-005</t>
         </is>
       </c>
       <c r="D31" s="13" t="inlineStr">
@@ -6068,7 +6071,7 @@
       </c>
       <c r="E31" s="10" t="inlineStr">
         <is>
-          <t>Consignment ops 200</t>
+          <t>Invalid/garbage token rejected</t>
         </is>
       </c>
     </row>
@@ -6080,12 +6083,12 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>Consignment</t>
+          <t>Auth &amp; Session</t>
         </is>
       </c>
       <c r="C32" s="10" t="inlineStr">
         <is>
-          <t>Web page renders: /consignment</t>
+          <t>Login (web UI) as SUPER_ADMIN</t>
         </is>
       </c>
       <c r="D32" s="13" t="inlineStr">
@@ -6095,7 +6098,7 @@
       </c>
       <c r="E32" s="10" t="inlineStr">
         <is>
-          <t>Rendered correctly; saw ["Consignment","Pulse"]</t>
+          <t>Logged in, redirected to app</t>
         </is>
       </c>
     </row>
@@ -6107,12 +6110,12 @@
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>Cross-Cutting Security, RBAC, Audit &amp; PCI</t>
+          <t>CIS &amp; Credit Onboarding</t>
         </is>
       </c>
       <c r="C33" s="10" t="inlineStr">
         <is>
-          <t>SEC-TC-001</t>
+          <t>CIS-TC-001</t>
         </is>
       </c>
       <c r="D33" s="13" t="inlineStr">
@@ -6122,7 +6125,7 @@
       </c>
       <c r="E33" s="10" t="inlineStr">
         <is>
-          <t>All sampled protected endpoints require authentication</t>
+          <t>FINANCE can read CIS finance queue</t>
         </is>
       </c>
     </row>
@@ -6134,12 +6137,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>Cross-Cutting Security, RBAC, Audit &amp; PCI</t>
+          <t>CIS &amp; Credit Onboarding</t>
         </is>
       </c>
       <c r="C34" s="10" t="inlineStr">
         <is>
-          <t>SEC-TC-002</t>
+          <t>CIS-TC-002</t>
         </is>
       </c>
       <c r="D34" s="13" t="inlineStr">
@@ -6149,7 +6152,7 @@
       </c>
       <c r="E34" s="10" t="inlineStr">
         <is>
-          <t>Default-deny: SALES_BD_REP denied admin module</t>
+          <t>TM denied CIS finance queue</t>
         </is>
       </c>
     </row>
@@ -6161,12 +6164,12 @@
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>Cross-Cutting Security, RBAC, Audit &amp; PCI</t>
+          <t>CIS &amp; Credit Onboarding</t>
         </is>
       </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>SEC-TC-010</t>
+          <t>CIS-TC-005</t>
         </is>
       </c>
       <c r="D35" s="13" t="inlineStr">
@@ -6176,7 +6179,7 @@
       </c>
       <c r="E35" s="10" t="inlineStr">
         <is>
-          <t>PCI guard rejects Luhn-valid PAN in lead note</t>
+          <t>CIS link blocked before discovery (server-enforced gate)</t>
         </is>
       </c>
     </row>
@@ -6188,12 +6191,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>Cross-Cutting Security, RBAC, Audit &amp; PCI</t>
+          <t>CIS &amp; Credit Onboarding</t>
         </is>
       </c>
       <c r="C36" s="10" t="inlineStr">
         <is>
-          <t>SEC-TC-011</t>
+          <t>CIS-TC-006</t>
         </is>
       </c>
       <c r="D36" s="13" t="inlineStr">
@@ -6203,7 +6206,7 @@
       </c>
       <c r="E36" s="10" t="inlineStr">
         <is>
-          <t>PCI guard does NOT false-positive on a 13-digit timestamp/order id</t>
+          <t>CIS link issued after discovery complete</t>
         </is>
       </c>
     </row>
@@ -6215,12 +6218,12 @@
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>Cross-Cutting Security, RBAC, Audit &amp; PCI</t>
+          <t>CIS &amp; Credit Onboarding</t>
         </is>
       </c>
       <c r="C37" s="10" t="inlineStr">
         <is>
-          <t>SEC-TC-020</t>
+          <t>CIS-TC-007</t>
         </is>
       </c>
       <c r="D37" s="13" t="inlineStr">
@@ -6230,24 +6233,24 @@
       </c>
       <c r="E37" s="10" t="inlineStr">
         <is>
-          <t>EXECUTIVE (read-only oversight) cannot mutate leads</t>
+          <t>TM denied CIS link issuance</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>WEB-UI</t>
         </is>
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>Dealer Portal &amp; Ordering</t>
+          <t>Calendar</t>
         </is>
       </c>
       <c r="C38" s="10" t="inlineStr">
         <is>
-          <t>DLR-TC-001</t>
+          <t>Web page renders: /calendar</t>
         </is>
       </c>
       <c r="D38" s="13" t="inlineStr">
@@ -6257,7 +6260,7 @@
       </c>
       <c r="E38" s="10" t="inlineStr">
         <is>
-          <t>Internal role cannot access dealer portal /me</t>
+          <t>Rendered correctly; saw ["Calendar","Pulse"]</t>
         </is>
       </c>
     </row>
@@ -6269,12 +6272,12 @@
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>Dealer Portal &amp; Ordering</t>
+          <t>Consignment</t>
         </is>
       </c>
       <c r="C39" s="10" t="inlineStr">
         <is>
-          <t>DLR-TC-002</t>
+          <t>CON-TC-001</t>
         </is>
       </c>
       <c r="D39" s="13" t="inlineStr">
@@ -6284,24 +6287,24 @@
       </c>
       <c r="E39" s="10" t="inlineStr">
         <is>
-          <t>Dealer /me catalog correctly unavailable to internal user (no dealer membership), got 400</t>
+          <t>Consignment sites 200</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="10" t="inlineStr">
         <is>
-          <t>WEB-UI</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>Dealer Portal &amp; Ordering</t>
+          <t>Consignment</t>
         </is>
       </c>
       <c r="C40" s="10" t="inlineStr">
         <is>
-          <t>Web page renders: /dealer/login</t>
+          <t>CON-TC-002</t>
         </is>
       </c>
       <c r="D40" s="13" t="inlineStr">
@@ -6311,7 +6314,7 @@
       </c>
       <c r="E40" s="10" t="inlineStr">
         <is>
-          <t>Rendered correctly; saw ["Dealer","Sign"]</t>
+          <t>Consignment dashboard 200</t>
         </is>
       </c>
     </row>
@@ -6323,12 +6326,12 @@
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>Digital Assets (DAM)</t>
+          <t>Consignment</t>
         </is>
       </c>
       <c r="C41" s="10" t="inlineStr">
         <is>
-          <t>DAM-TC-001</t>
+          <t>CON-TC-003</t>
         </is>
       </c>
       <c r="D41" s="13" t="inlineStr">
@@ -6338,7 +6341,7 @@
       </c>
       <c r="E41" s="10" t="inlineStr">
         <is>
-          <t>DAM assets 200</t>
+          <t>Consignment ops 200</t>
         </is>
       </c>
     </row>
@@ -6350,12 +6353,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>Digital Assets (DAM)</t>
+          <t>Consignment</t>
         </is>
       </c>
       <c r="C42" s="10" t="inlineStr">
         <is>
-          <t>DAM-TC-002</t>
+          <t>CON-TC-010</t>
         </is>
       </c>
       <c r="D42" s="13" t="inlineStr">
@@ -6365,24 +6368,24 @@
       </c>
       <c r="E42" s="10" t="inlineStr">
         <is>
-          <t>DAM collections 200</t>
+          <t>Create consignment site</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="10" t="inlineStr">
         <is>
-          <t>WEB-UI</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t>Digital Assets (DAM)</t>
+          <t>Consignment</t>
         </is>
       </c>
       <c r="C43" s="10" t="inlineStr">
         <is>
-          <t>Web page renders: /digital-assets</t>
+          <t>CON-TC-011</t>
         </is>
       </c>
       <c r="D43" s="13" t="inlineStr">
@@ -6392,24 +6395,24 @@
       </c>
       <c r="E43" s="10" t="inlineStr">
         <is>
-          <t>Rendered correctly; saw ["Digital Assets","Library"]</t>
+          <t>Consignment site detail</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>WEB-UI</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>Digital Assets (DAM)</t>
+          <t>Consignment</t>
         </is>
       </c>
       <c r="C44" s="10" t="inlineStr">
         <is>
-          <t>Web page renders: /digital-assets?tab=migration</t>
+          <t>CON-TC-012</t>
         </is>
       </c>
       <c r="D44" s="13" t="inlineStr">
@@ -6419,7 +6422,7 @@
       </c>
       <c r="E44" s="10" t="inlineStr">
         <is>
-          <t>Rendered correctly; saw ["Migration Review","Widen"]</t>
+          <t>Consignment readiness</t>
         </is>
       </c>
     </row>
@@ -6431,12 +6434,12 @@
       </c>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Consignment</t>
         </is>
       </c>
       <c r="C45" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-005</t>
+          <t>CON-TC-013</t>
         </is>
       </c>
       <c r="D45" s="13" t="inlineStr">
@@ -6446,7 +6449,7 @@
       </c>
       <c r="E45" s="10" t="inlineStr">
         <is>
-          <t>Authorized user created a manual lead</t>
+          <t>Consignment documents</t>
         </is>
       </c>
     </row>
@@ -6458,12 +6461,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Consignment</t>
         </is>
       </c>
       <c r="C46" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-006a</t>
+          <t>CON-TC-014</t>
         </is>
       </c>
       <c r="D46" s="13" t="inlineStr">
@@ -6473,7 +6476,7 @@
       </c>
       <c r="E46" s="10" t="inlineStr">
         <is>
-          <t>TERRITORY_MANAGER correctly denied lead creation (default-deny)</t>
+          <t>Create consignment audit</t>
         </is>
       </c>
     </row>
@@ -6485,39 +6488,39 @@
       </c>
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Consignment</t>
         </is>
       </c>
       <c r="C47" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-006b</t>
-        </is>
-      </c>
-      <c r="D47" s="13" t="inlineStr">
-        <is>
-          <t>PASS</t>
+          <t>CON-TC-031</t>
+        </is>
+      </c>
+      <c r="D47" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="E47" s="10" t="inlineStr">
         <is>
-          <t>REGIONAL_DIRECTOR correctly denied lead creation (default-deny)</t>
+          <t>DEFECT — consignment-site note ACCEPTED + stored a raw card number (HTTP 201); PCI guard not enforced on consignment notes in the deployed build (fix 327b6e9 not deployed). Leads/CIS reject the same input; consignment does not.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="10" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>WEB-UI</t>
         </is>
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Consignment</t>
         </is>
       </c>
       <c r="C48" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-006c</t>
+          <t>Web page renders: /consignment</t>
         </is>
       </c>
       <c r="D48" s="13" t="inlineStr">
@@ -6527,7 +6530,7 @@
       </c>
       <c r="E48" s="10" t="inlineStr">
         <is>
-          <t>FINANCE correctly denied lead creation (default-deny)</t>
+          <t>Rendered correctly; saw ["Consignment","Pulse"]</t>
         </is>
       </c>
     </row>
@@ -6539,12 +6542,12 @@
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Cross-Cutting Security, RBAC, Audit &amp; PCI</t>
         </is>
       </c>
       <c r="C49" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-007</t>
+          <t>SEC-TC-001</t>
         </is>
       </c>
       <c r="D49" s="13" t="inlineStr">
@@ -6554,7 +6557,7 @@
       </c>
       <c r="E49" s="10" t="inlineStr">
         <is>
-          <t>Invalid email rejected at intake</t>
+          <t>All sampled protected endpoints require authentication</t>
         </is>
       </c>
     </row>
@@ -6566,12 +6569,12 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Cross-Cutting Security, RBAC, Audit &amp; PCI</t>
         </is>
       </c>
       <c r="C50" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-008</t>
+          <t>SEC-TC-002</t>
         </is>
       </c>
       <c r="D50" s="13" t="inlineStr">
@@ -6581,7 +6584,7 @@
       </c>
       <c r="E50" s="10" t="inlineStr">
         <is>
-          <t>Invalid phone (too few digits) rejected</t>
+          <t>Default-deny: SALES_BD_REP denied admin module</t>
         </is>
       </c>
     </row>
@@ -6593,12 +6596,12 @@
       </c>
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Cross-Cutting Security, RBAC, Audit &amp; PCI</t>
         </is>
       </c>
       <c r="C51" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-009</t>
+          <t>SEC-TC-010</t>
         </is>
       </c>
       <c r="D51" s="13" t="inlineStr">
@@ -6608,7 +6611,7 @@
       </c>
       <c r="E51" s="10" t="inlineStr">
         <is>
-          <t>Missing company rejected</t>
+          <t>PCI guard rejects Luhn-valid PAN in lead note</t>
         </is>
       </c>
     </row>
@@ -6620,12 +6623,12 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Cross-Cutting Security, RBAC, Audit &amp; PCI</t>
         </is>
       </c>
       <c r="C52" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-031</t>
+          <t>SEC-TC-011</t>
         </is>
       </c>
       <c r="D52" s="13" t="inlineStr">
@@ -6635,7 +6638,7 @@
       </c>
       <c r="E52" s="10" t="inlineStr">
         <is>
-          <t>PCI: raw card number in lead note rejected</t>
+          <t>PCI guard does NOT false-positive on a 13-digit timestamp/order id</t>
         </is>
       </c>
     </row>
@@ -6647,12 +6650,12 @@
       </c>
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Cross-Cutting Security, RBAC, Audit &amp; PCI</t>
         </is>
       </c>
       <c r="C53" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-040</t>
+          <t>SEC-TC-020</t>
         </is>
       </c>
       <c r="D53" s="13" t="inlineStr">
@@ -6662,7 +6665,7 @@
       </c>
       <c r="E53" s="10" t="inlineStr">
         <is>
-          <t>Lead list returns items</t>
+          <t>EXECUTIVE (read-only oversight) cannot mutate leads</t>
         </is>
       </c>
     </row>
@@ -6674,12 +6677,12 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Dealer Portal &amp; Ordering</t>
         </is>
       </c>
       <c r="C54" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-041</t>
+          <t>DLR-TC-001</t>
         </is>
       </c>
       <c r="D54" s="13" t="inlineStr">
@@ -6689,7 +6692,7 @@
       </c>
       <c r="E54" s="10" t="inlineStr">
         <is>
-          <t>Non-existent lead returns not-found/forbidden</t>
+          <t>Internal role cannot access dealer portal /me</t>
         </is>
       </c>
     </row>
@@ -6701,12 +6704,12 @@
       </c>
       <c r="B55" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Dealer Portal &amp; Ordering</t>
         </is>
       </c>
       <c r="C55" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-053</t>
+          <t>DLR-TC-002</t>
         </is>
       </c>
       <c r="D55" s="13" t="inlineStr">
@@ -6716,24 +6719,24 @@
       </c>
       <c r="E55" s="10" t="inlineStr">
         <is>
-          <t>Duplicate detection: 2nd lead with same phone is blocked pending resolution (400)</t>
+          <t>Dealer /me catalog correctly unavailable to internal user (no dealer membership), got 400</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="10" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>WEB-UI</t>
         </is>
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Dealer Portal &amp; Ordering</t>
         </is>
       </c>
       <c r="C56" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-008b</t>
+          <t>Web page renders: /dealer/login</t>
         </is>
       </c>
       <c r="D56" s="13" t="inlineStr">
@@ -6743,7 +6746,7 @@
       </c>
       <c r="E56" s="10" t="inlineStr">
         <is>
-          <t>7-digit phone (lower boundary) accepted</t>
+          <t>Rendered correctly; saw ["Dealer","Sign"]</t>
         </is>
       </c>
     </row>
@@ -6755,12 +6758,12 @@
       </c>
       <c r="B57" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Digital Assets (DAM)</t>
         </is>
       </c>
       <c r="C57" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-008c</t>
+          <t>DAM-TC-001</t>
         </is>
       </c>
       <c r="D57" s="13" t="inlineStr">
@@ -6770,7 +6773,7 @@
       </c>
       <c r="E57" s="10" t="inlineStr">
         <is>
-          <t>16-digit phone (over boundary) rejected</t>
+          <t>DAM assets 200</t>
         </is>
       </c>
     </row>
@@ -6782,12 +6785,12 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Digital Assets (DAM)</t>
         </is>
       </c>
       <c r="C58" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-050</t>
+          <t>DAM-TC-002</t>
         </is>
       </c>
       <c r="D58" s="13" t="inlineStr">
@@ -6797,7 +6800,7 @@
       </c>
       <c r="E58" s="10" t="inlineStr">
         <is>
-          <t>Special chars / SQL-ish input handled without server error</t>
+          <t>DAM collections 200</t>
         </is>
       </c>
     </row>
@@ -6809,12 +6812,12 @@
       </c>
       <c r="B59" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Digital Assets (DAM)</t>
         </is>
       </c>
       <c r="C59" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-051</t>
+          <t>DAM-TC-011</t>
         </is>
       </c>
       <c r="D59" s="13" t="inlineStr">
@@ -6824,7 +6827,7 @@
       </c>
       <c r="E59" s="10" t="inlineStr">
         <is>
-          <t>Oversized field handled gracefully (400)</t>
+          <t>DAM Widen import runs list</t>
         </is>
       </c>
     </row>
@@ -6836,12 +6839,12 @@
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Digital Assets (DAM)</t>
         </is>
       </c>
       <c r="C60" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-052</t>
+          <t>DAM-TC-012</t>
         </is>
       </c>
       <c r="D60" s="13" t="inlineStr">
@@ -6851,24 +6854,24 @@
       </c>
       <c r="E60" s="10" t="inlineStr">
         <is>
-          <t>Pagination limit honoured (&lt;=2 items)</t>
+          <t>DAM Widen import preview endpoint reachable (405)</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="10" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>WEB-UI</t>
         </is>
       </c>
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Digital Assets (DAM)</t>
         </is>
       </c>
       <c r="C61" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-020</t>
+          <t>Web page renders: /digital-assets</t>
         </is>
       </c>
       <c r="D61" s="13" t="inlineStr">
@@ -6878,24 +6881,24 @@
       </c>
       <c r="E61" s="10" t="inlineStr">
         <is>
-          <t>Discovery scheduled</t>
+          <t>Rendered correctly; saw ["Digital Assets","Library"]</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="10" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>WEB-UI</t>
         </is>
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Digital Assets (DAM)</t>
         </is>
       </c>
       <c r="C62" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-021</t>
+          <t>Web page renders: /digital-assets?tab=migration</t>
         </is>
       </c>
       <c r="D62" s="13" t="inlineStr">
@@ -6905,14 +6908,14 @@
       </c>
       <c r="E62" s="10" t="inlineStr">
         <is>
-          <t>Discovery completed (lead advanced)</t>
+          <t>Rendered correctly; saw ["Migration Review","Widen"]</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="10" t="inlineStr">
         <is>
-          <t>WEB-UI</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B63" s="10" t="inlineStr">
@@ -6922,7 +6925,7 @@
       </c>
       <c r="C63" s="10" t="inlineStr">
         <is>
-          <t>Leads: list renders rows</t>
+          <t>LEAD-TC-005</t>
         </is>
       </c>
       <c r="D63" s="13" t="inlineStr">
@@ -6932,14 +6935,14 @@
       </c>
       <c r="E63" s="10" t="inlineStr">
         <is>
-          <t>104 lead rows/links present</t>
+          <t>Authorized user created a manual lead</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="10" t="inlineStr">
         <is>
-          <t>WEB-UI</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B64" s="10" t="inlineStr">
@@ -6949,7 +6952,7 @@
       </c>
       <c r="C64" s="10" t="inlineStr">
         <is>
-          <t>Web page renders: /leads</t>
+          <t>LEAD-TC-006a</t>
         </is>
       </c>
       <c r="D64" s="13" t="inlineStr">
@@ -6959,7 +6962,7 @@
       </c>
       <c r="E64" s="10" t="inlineStr">
         <is>
-          <t>Rendered correctly; saw ["Lead","QA-HVAC"]</t>
+          <t>TERRITORY_MANAGER correctly denied lead creation (default-deny)</t>
         </is>
       </c>
     </row>
@@ -6971,12 +6974,12 @@
       </c>
       <c r="B65" s="10" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C65" s="10" t="inlineStr">
         <is>
-          <t>NOT-TC-001</t>
+          <t>LEAD-TC-006b</t>
         </is>
       </c>
       <c r="D65" s="13" t="inlineStr">
@@ -6986,7 +6989,7 @@
       </c>
       <c r="E65" s="10" t="inlineStr">
         <is>
-          <t>Notifications inbox list 200</t>
+          <t>REGIONAL_DIRECTOR correctly denied lead creation (default-deny)</t>
         </is>
       </c>
     </row>
@@ -6998,12 +7001,12 @@
       </c>
       <c r="B66" s="10" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C66" s="10" t="inlineStr">
         <is>
-          <t>NOT-TC-002</t>
+          <t>LEAD-TC-006c</t>
         </is>
       </c>
       <c r="D66" s="13" t="inlineStr">
@@ -7013,7 +7016,7 @@
       </c>
       <c r="E66" s="10" t="inlineStr">
         <is>
-          <t>Notifications unread count 200</t>
+          <t>FINANCE correctly denied lead creation (default-deny)</t>
         </is>
       </c>
     </row>
@@ -7025,12 +7028,12 @@
       </c>
       <c r="B67" s="10" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C67" s="10" t="inlineStr">
         <is>
-          <t>NOT-TC-003</t>
+          <t>LEAD-TC-007</t>
         </is>
       </c>
       <c r="D67" s="13" t="inlineStr">
@@ -7040,7 +7043,7 @@
       </c>
       <c r="E67" s="10" t="inlineStr">
         <is>
-          <t>Notifications preferences 200</t>
+          <t>Invalid email rejected at intake</t>
         </is>
       </c>
     </row>
@@ -7052,12 +7055,12 @@
       </c>
       <c r="B68" s="10" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C68" s="10" t="inlineStr">
         <is>
-          <t>NOT-TC-010</t>
+          <t>LEAD-TC-008</t>
         </is>
       </c>
       <c r="D68" s="13" t="inlineStr">
@@ -7067,7 +7070,7 @@
       </c>
       <c r="E68" s="10" t="inlineStr">
         <is>
-          <t>Admin can read routing rules</t>
+          <t>Invalid phone (too few digits) rejected</t>
         </is>
       </c>
     </row>
@@ -7079,12 +7082,12 @@
       </c>
       <c r="B69" s="10" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C69" s="10" t="inlineStr">
         <is>
-          <t>NOT-TC-011</t>
+          <t>LEAD-TC-009</t>
         </is>
       </c>
       <c r="D69" s="13" t="inlineStr">
@@ -7094,24 +7097,24 @@
       </c>
       <c r="E69" s="10" t="inlineStr">
         <is>
-          <t>Routing rules access for TM controlled (403)</t>
+          <t>Missing company rejected</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="10" t="inlineStr">
         <is>
-          <t>WEB-UI</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B70" s="10" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C70" s="10" t="inlineStr">
         <is>
-          <t>Web page renders: /notifications</t>
+          <t>LEAD-TC-031</t>
         </is>
       </c>
       <c r="D70" s="13" t="inlineStr">
@@ -7121,24 +7124,24 @@
       </c>
       <c r="E70" s="10" t="inlineStr">
         <is>
-          <t>Rendered correctly; saw ["Notifications"]</t>
+          <t>PCI: raw card number in lead note rejected</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="10" t="inlineStr">
         <is>
-          <t>WEB-UI</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B71" s="10" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C71" s="10" t="inlineStr">
         <is>
-          <t>Web page renders: /settings/notifications/routing</t>
+          <t>LEAD-TC-040</t>
         </is>
       </c>
       <c r="D71" s="13" t="inlineStr">
@@ -7148,24 +7151,24 @@
       </c>
       <c r="E71" s="10" t="inlineStr">
         <is>
-          <t>Rendered correctly; saw ["Recipient"]</t>
+          <t>Lead list returns items</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="10" t="inlineStr">
         <is>
-          <t>WEB-UI</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B72" s="10" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C72" s="10" t="inlineStr">
         <is>
-          <t>Web page renders: /settings/notifications</t>
+          <t>LEAD-TC-041</t>
         </is>
       </c>
       <c r="D72" s="13" t="inlineStr">
@@ -7175,7 +7178,7 @@
       </c>
       <c r="E72" s="10" t="inlineStr">
         <is>
-          <t>Rendered correctly; saw ["Notification preferences"]</t>
+          <t>Non-existent lead returns not-found/forbidden</t>
         </is>
       </c>
     </row>
@@ -7187,12 +7190,12 @@
       </c>
       <c r="B73" s="10" t="inlineStr">
         <is>
-          <t>Product Management &amp; Catalog</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C73" s="10" t="inlineStr">
         <is>
-          <t>PM-TC-001</t>
+          <t>LEAD-TC-053</t>
         </is>
       </c>
       <c r="D73" s="13" t="inlineStr">
@@ -7202,7 +7205,7 @@
       </c>
       <c r="E73" s="10" t="inlineStr">
         <is>
-          <t>Product families 200</t>
+          <t>Duplicate detection: 2nd lead with same phone is blocked pending resolution (400)</t>
         </is>
       </c>
     </row>
@@ -7214,12 +7217,12 @@
       </c>
       <c r="B74" s="10" t="inlineStr">
         <is>
-          <t>Product Management &amp; Catalog</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C74" s="10" t="inlineStr">
         <is>
-          <t>PM-TC-002</t>
+          <t>LEAD-TC-008b</t>
         </is>
       </c>
       <c r="D74" s="13" t="inlineStr">
@@ -7229,7 +7232,7 @@
       </c>
       <c r="E74" s="10" t="inlineStr">
         <is>
-          <t>Product categories 200</t>
+          <t>7-digit phone (lower boundary) accepted</t>
         </is>
       </c>
     </row>
@@ -7241,12 +7244,12 @@
       </c>
       <c r="B75" s="10" t="inlineStr">
         <is>
-          <t>Product Management &amp; Catalog</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C75" s="10" t="inlineStr">
         <is>
-          <t>PM-TC-003</t>
+          <t>LEAD-TC-008c</t>
         </is>
       </c>
       <c r="D75" s="13" t="inlineStr">
@@ -7256,7 +7259,7 @@
       </c>
       <c r="E75" s="10" t="inlineStr">
         <is>
-          <t>Product rule sets 200</t>
+          <t>16-digit phone (over boundary) rejected</t>
         </is>
       </c>
     </row>
@@ -7268,12 +7271,12 @@
       </c>
       <c r="B76" s="10" t="inlineStr">
         <is>
-          <t>Product Management &amp; Catalog</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C76" s="10" t="inlineStr">
         <is>
-          <t>PM-TC-004</t>
+          <t>LEAD-TC-050</t>
         </is>
       </c>
       <c r="D76" s="13" t="inlineStr">
@@ -7283,24 +7286,24 @@
       </c>
       <c r="E76" s="10" t="inlineStr">
         <is>
-          <t>Product catalog views 200</t>
+          <t>Special chars / SQL-ish input handled without server error</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="10" t="inlineStr">
         <is>
-          <t>WEB-UI</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B77" s="10" t="inlineStr">
         <is>
-          <t>Product Management &amp; Catalog</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C77" s="10" t="inlineStr">
         <is>
-          <t>Web page renders: /product-management</t>
+          <t>LEAD-TC-051</t>
         </is>
       </c>
       <c r="D77" s="13" t="inlineStr">
@@ -7310,7 +7313,7 @@
       </c>
       <c r="E77" s="10" t="inlineStr">
         <is>
-          <t>Rendered correctly; saw ["Product","Pulse"]</t>
+          <t>Oversized field handled gracefully (400)</t>
         </is>
       </c>
     </row>
@@ -7322,12 +7325,12 @@
       </c>
       <c r="B78" s="10" t="inlineStr">
         <is>
-          <t>Reporting &amp; Dashboards</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C78" s="10" t="inlineStr">
         <is>
-          <t>RPT-TC-001</t>
+          <t>LEAD-TC-052</t>
         </is>
       </c>
       <c r="D78" s="13" t="inlineStr">
@@ -7337,7 +7340,7 @@
       </c>
       <c r="E78" s="10" t="inlineStr">
         <is>
-          <t>Lead dashboard returns 200 for SUPER_ADMIN</t>
+          <t>Pagination limit honoured (&lt;=2 items)</t>
         </is>
       </c>
     </row>
@@ -7349,12 +7352,12 @@
       </c>
       <c r="B79" s="10" t="inlineStr">
         <is>
-          <t>Reporting &amp; Dashboards</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C79" s="10" t="inlineStr">
         <is>
-          <t>RPT-TC-002</t>
+          <t>LEAD-TC-020</t>
         </is>
       </c>
       <c r="D79" s="13" t="inlineStr">
@@ -7364,7 +7367,7 @@
       </c>
       <c r="E79" s="10" t="inlineStr">
         <is>
-          <t>Training dashboard returns 200 for SUPER_ADMIN</t>
+          <t>Discovery scheduled</t>
         </is>
       </c>
     </row>
@@ -7376,12 +7379,12 @@
       </c>
       <c r="B80" s="10" t="inlineStr">
         <is>
-          <t>Reporting &amp; Dashboards</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C80" s="10" t="inlineStr">
         <is>
-          <t>RPT-TC-003</t>
+          <t>LEAD-TC-021</t>
         </is>
       </c>
       <c r="D80" s="13" t="inlineStr">
@@ -7391,7 +7394,7 @@
       </c>
       <c r="E80" s="10" t="inlineStr">
         <is>
-          <t>Executive dashboard returns 200 for SUPER_ADMIN</t>
+          <t>Discovery completed (lead advanced)</t>
         </is>
       </c>
     </row>
@@ -7403,12 +7406,12 @@
       </c>
       <c r="B81" s="10" t="inlineStr">
         <is>
-          <t>Reporting &amp; Dashboards</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C81" s="10" t="inlineStr">
         <is>
-          <t>RPT-TC-020</t>
+          <t>LEAD-TC-002b</t>
         </is>
       </c>
       <c r="D81" s="13" t="inlineStr">
@@ -7418,7 +7421,7 @@
       </c>
       <c r="E81" s="10" t="inlineStr">
         <is>
-          <t>EXECUTIVE can view executive dashboard</t>
+          <t>Create lead (deep fixture)</t>
         </is>
       </c>
     </row>
@@ -7430,12 +7433,12 @@
       </c>
       <c r="B82" s="10" t="inlineStr">
         <is>
-          <t>Reporting &amp; Dashboards</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C82" s="10" t="inlineStr">
         <is>
-          <t>RPT-TC-021</t>
+          <t>LEAD-TC-060</t>
         </is>
       </c>
       <c r="D82" s="13" t="inlineStr">
@@ -7445,7 +7448,7 @@
       </c>
       <c r="E82" s="10" t="inlineStr">
         <is>
-          <t>TM denied executive dashboard (reports.executive gate)</t>
+          <t>Add lead contact</t>
         </is>
       </c>
     </row>
@@ -7457,12 +7460,12 @@
       </c>
       <c r="B83" s="10" t="inlineStr">
         <is>
-          <t>Reporting &amp; Dashboards</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C83" s="10" t="inlineStr">
         <is>
-          <t>RPT-TC-039</t>
+          <t>LEAD-TC-061</t>
         </is>
       </c>
       <c r="D83" s="13" t="inlineStr">
@@ -7472,7 +7475,7 @@
       </c>
       <c r="E83" s="10" t="inlineStr">
         <is>
-          <t>Stale/neglected accounts report 200</t>
+          <t>List lead contacts</t>
         </is>
       </c>
     </row>
@@ -7484,12 +7487,12 @@
       </c>
       <c r="B84" s="10" t="inlineStr">
         <is>
-          <t>Reporting &amp; Dashboards</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C84" s="10" t="inlineStr">
         <is>
-          <t>RPT-TC-003b</t>
+          <t>LEAD-TC-062</t>
         </is>
       </c>
       <c r="D84" s="13" t="inlineStr">
@@ -7499,7 +7502,7 @@
       </c>
       <c r="E84" s="10" t="inlineStr">
         <is>
-          <t>Threshold settings readable</t>
+          <t>Log activity note</t>
         </is>
       </c>
     </row>
@@ -7511,12 +7514,12 @@
       </c>
       <c r="B85" s="10" t="inlineStr">
         <is>
-          <t>Reporting &amp; Dashboards</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C85" s="10" t="inlineStr">
         <is>
-          <t>RPT-TC-022b</t>
+          <t>LEAD-TC-070</t>
         </is>
       </c>
       <c r="D85" s="13" t="inlineStr">
@@ -7526,24 +7529,24 @@
       </c>
       <c r="E85" s="10" t="inlineStr">
         <is>
-          <t>TM threshold-settings access controlled (200)</t>
+          <t>Lead readiness loads</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="10" t="inlineStr">
         <is>
-          <t>WEB-UI</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B86" s="10" t="inlineStr">
         <is>
-          <t>Reporting &amp; Dashboards</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C86" s="10" t="inlineStr">
         <is>
-          <t>Reports: dashboard Export control present (CSV/Excel/PDF)</t>
+          <t>LEAD-TC-072</t>
         </is>
       </c>
       <c r="D86" s="13" t="inlineStr">
@@ -7553,24 +7556,24 @@
       </c>
       <c r="E86" s="10" t="inlineStr">
         <is>
-          <t>Export button rendered on dashboard</t>
+          <t>Lead readiness blockers loads</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="10" t="inlineStr">
         <is>
-          <t>WEB-UI</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B87" s="10" t="inlineStr">
         <is>
-          <t>Reporting &amp; Dashboards</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C87" s="10" t="inlineStr">
         <is>
-          <t>Web page renders: /reports</t>
+          <t>LEAD-TC-073</t>
         </is>
       </c>
       <c r="D87" s="13" t="inlineStr">
@@ -7580,7 +7583,7 @@
       </c>
       <c r="E87" s="10" t="inlineStr">
         <is>
-          <t>Rendered correctly; saw ["Reports","Export"]</t>
+          <t>Log initial contact</t>
         </is>
       </c>
     </row>
@@ -7592,12 +7595,12 @@
       </c>
       <c r="B88" s="10" t="inlineStr">
         <is>
-          <t>Territory</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C88" s="10" t="inlineStr">
         <is>
-          <t>TER-TC-001</t>
+          <t>LEAD-TC-074</t>
         </is>
       </c>
       <c r="D88" s="13" t="inlineStr">
@@ -7607,7 +7610,7 @@
       </c>
       <c r="E88" s="10" t="inlineStr">
         <is>
-          <t>Territory list 200</t>
+          <t>Lead search filter</t>
         </is>
       </c>
     </row>
@@ -7619,12 +7622,12 @@
       </c>
       <c r="B89" s="10" t="inlineStr">
         <is>
-          <t>Territory</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C89" s="10" t="inlineStr">
         <is>
-          <t>TER-TC-002</t>
+          <t>LEAD-TC-075</t>
         </is>
       </c>
       <c r="D89" s="13" t="inlineStr">
@@ -7634,7 +7637,7 @@
       </c>
       <c r="E89" s="10" t="inlineStr">
         <is>
-          <t>Territory regions 200</t>
+          <t>Lead stage filter</t>
         </is>
       </c>
     </row>
@@ -7646,12 +7649,12 @@
       </c>
       <c r="B90" s="10" t="inlineStr">
         <is>
-          <t>Territory</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C90" s="10" t="inlineStr">
         <is>
-          <t>TER-TC-003</t>
+          <t>LEAD-TC-076</t>
         </is>
       </c>
       <c r="D90" s="13" t="inlineStr">
@@ -7661,24 +7664,24 @@
       </c>
       <c r="E90" s="10" t="inlineStr">
         <is>
-          <t>Territory map 200</t>
+          <t>TM can view leads (scoped)</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="10" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>WEB-UI</t>
         </is>
       </c>
       <c r="B91" s="10" t="inlineStr">
         <is>
-          <t>Territory</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C91" s="10" t="inlineStr">
         <is>
-          <t>TER-TC-004</t>
+          <t>Leads: list renders rows</t>
         </is>
       </c>
       <c r="D91" s="13" t="inlineStr">
@@ -7688,24 +7691,24 @@
       </c>
       <c r="E91" s="10" t="inlineStr">
         <is>
-          <t>Territory dashboard 200</t>
+          <t>104 lead rows/links present</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="10" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>WEB-UI</t>
         </is>
       </c>
       <c r="B92" s="10" t="inlineStr">
         <is>
-          <t>Territory</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C92" s="10" t="inlineStr">
         <is>
-          <t>TER-TC-010</t>
+          <t>Web page renders: /leads</t>
         </is>
       </c>
       <c r="D92" s="13" t="inlineStr">
@@ -7715,24 +7718,24 @@
       </c>
       <c r="E92" s="10" t="inlineStr">
         <is>
-          <t>TM can read territories</t>
+          <t>Rendered correctly; saw ["Lead","QA-HVAC"]</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="10" t="inlineStr">
         <is>
-          <t>WEB-UI</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B93" s="10" t="inlineStr">
         <is>
-          <t>Territory</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C93" s="10" t="inlineStr">
         <is>
-          <t>Web page renders: /territories</t>
+          <t>NOT-TC-001</t>
         </is>
       </c>
       <c r="D93" s="13" t="inlineStr">
@@ -7742,24 +7745,24 @@
       </c>
       <c r="E93" s="10" t="inlineStr">
         <is>
-          <t>Rendered correctly; saw ["Territor","Pulse"]</t>
+          <t>Notifications inbox list 200</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="10" t="inlineStr">
         <is>
-          <t>WEB-UI</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B94" s="10" t="inlineStr">
         <is>
-          <t>Territory</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C94" s="10" t="inlineStr">
         <is>
-          <t>Web page renders: /territory_map</t>
+          <t>NOT-TC-002</t>
         </is>
       </c>
       <c r="D94" s="13" t="inlineStr">
@@ -7769,7 +7772,7 @@
       </c>
       <c r="E94" s="10" t="inlineStr">
         <is>
-          <t>Rendered correctly; saw ["Pulse"]</t>
+          <t>Notifications unread count 200</t>
         </is>
       </c>
     </row>
@@ -7781,12 +7784,12 @@
       </c>
       <c r="B95" s="10" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C95" s="10" t="inlineStr">
         <is>
-          <t>TRN-TC-001</t>
+          <t>NOT-TC-003</t>
         </is>
       </c>
       <c r="D95" s="13" t="inlineStr">
@@ -7796,7 +7799,7 @@
       </c>
       <c r="E95" s="10" t="inlineStr">
         <is>
-          <t>Training sessions 200</t>
+          <t>Notifications preferences 200</t>
         </is>
       </c>
     </row>
@@ -7808,12 +7811,12 @@
       </c>
       <c r="B96" s="10" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C96" s="10" t="inlineStr">
         <is>
-          <t>TRN-TC-002</t>
+          <t>NOT-TC-010</t>
         </is>
       </c>
       <c r="D96" s="13" t="inlineStr">
@@ -7823,7 +7826,7 @@
       </c>
       <c r="E96" s="10" t="inlineStr">
         <is>
-          <t>Training overview 200</t>
+          <t>Admin can read routing rules</t>
         </is>
       </c>
     </row>
@@ -7835,12 +7838,12 @@
       </c>
       <c r="B97" s="10" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C97" s="10" t="inlineStr">
         <is>
-          <t>TRN-TC-003</t>
+          <t>NOT-TC-011</t>
         </is>
       </c>
       <c r="D97" s="13" t="inlineStr">
@@ -7850,7 +7853,7 @@
       </c>
       <c r="E97" s="10" t="inlineStr">
         <is>
-          <t>Training catalog 200</t>
+          <t>Routing rules access for TM controlled (403)</t>
         </is>
       </c>
     </row>
@@ -7862,12 +7865,12 @@
       </c>
       <c r="B98" s="10" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C98" s="10" t="inlineStr">
         <is>
-          <t>TRN-TC-004</t>
+          <t>NOT-TC-020</t>
         </is>
       </c>
       <c r="D98" s="13" t="inlineStr">
@@ -7877,7 +7880,7 @@
       </c>
       <c r="E98" s="10" t="inlineStr">
         <is>
-          <t>Training trainers 200</t>
+          <t>Mark notifications read</t>
         </is>
       </c>
     </row>
@@ -7889,54 +7892,1296 @@
       </c>
       <c r="B99" s="10" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C99" s="10" t="inlineStr">
         <is>
-          <t>TRN-TC-010</t>
-        </is>
-      </c>
-      <c r="D99" s="13" t="inlineStr">
-        <is>
-          <t>PASS</t>
+          <t>NOT-TC-021</t>
+        </is>
+      </c>
+      <c r="D99" s="14" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="E99" s="10" t="inlineStr">
         <is>
-          <t>TRAINING_OPS can read sessions</t>
+          <t>400: A valid notification category is required.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="10" t="inlineStr">
         <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B100" s="10" t="inlineStr">
+        <is>
+          <t>Notifications</t>
+        </is>
+      </c>
+      <c r="C100" s="10" t="inlineStr">
+        <is>
+          <t>NOT-TC-022</t>
+        </is>
+      </c>
+      <c r="D100" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E100" s="10" t="inlineStr">
+        <is>
+          <t>Create notification routing rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B101" s="10" t="inlineStr">
+        <is>
+          <t>Notifications</t>
+        </is>
+      </c>
+      <c r="C101" s="10" t="inlineStr">
+        <is>
+          <t>NOT-TC-023</t>
+        </is>
+      </c>
+      <c r="D101" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E101" s="10" t="inlineStr">
+        <is>
+          <t>Delete routing rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B102" s="10" t="inlineStr">
+        <is>
+          <t>Notifications</t>
+        </is>
+      </c>
+      <c r="C102" s="10" t="inlineStr">
+        <is>
+          <t>NOT-TC-024</t>
+        </is>
+      </c>
+      <c r="D102" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E102" s="10" t="inlineStr">
+        <is>
+          <t>TM denied routing-rule creation (admin-gated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="10" t="inlineStr">
+        <is>
           <t>WEB-UI</t>
         </is>
       </c>
-      <c r="B100" s="10" t="inlineStr">
+      <c r="B103" s="10" t="inlineStr">
+        <is>
+          <t>Notifications</t>
+        </is>
+      </c>
+      <c r="C103" s="10" t="inlineStr">
+        <is>
+          <t>Web page renders: /notifications</t>
+        </is>
+      </c>
+      <c r="D103" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E103" s="10" t="inlineStr">
+        <is>
+          <t>Rendered correctly; saw ["Notifications"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="10" t="inlineStr">
+        <is>
+          <t>WEB-UI</t>
+        </is>
+      </c>
+      <c r="B104" s="10" t="inlineStr">
+        <is>
+          <t>Notifications</t>
+        </is>
+      </c>
+      <c r="C104" s="10" t="inlineStr">
+        <is>
+          <t>Web page renders: /settings/notifications/routing</t>
+        </is>
+      </c>
+      <c r="D104" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E104" s="10" t="inlineStr">
+        <is>
+          <t>Rendered correctly; saw ["Recipient"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="10" t="inlineStr">
+        <is>
+          <t>WEB-UI</t>
+        </is>
+      </c>
+      <c r="B105" s="10" t="inlineStr">
+        <is>
+          <t>Notifications</t>
+        </is>
+      </c>
+      <c r="C105" s="10" t="inlineStr">
+        <is>
+          <t>Web page renders: /settings/notifications</t>
+        </is>
+      </c>
+      <c r="D105" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E105" s="10" t="inlineStr">
+        <is>
+          <t>Rendered correctly; saw ["Notification preferences"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B106" s="10" t="inlineStr">
+        <is>
+          <t>Product Management &amp; Catalog</t>
+        </is>
+      </c>
+      <c r="C106" s="10" t="inlineStr">
+        <is>
+          <t>PM-TC-001</t>
+        </is>
+      </c>
+      <c r="D106" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E106" s="10" t="inlineStr">
+        <is>
+          <t>Product families 200</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B107" s="10" t="inlineStr">
+        <is>
+          <t>Product Management &amp; Catalog</t>
+        </is>
+      </c>
+      <c r="C107" s="10" t="inlineStr">
+        <is>
+          <t>PM-TC-002</t>
+        </is>
+      </c>
+      <c r="D107" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E107" s="10" t="inlineStr">
+        <is>
+          <t>Product categories 200</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B108" s="10" t="inlineStr">
+        <is>
+          <t>Product Management &amp; Catalog</t>
+        </is>
+      </c>
+      <c r="C108" s="10" t="inlineStr">
+        <is>
+          <t>PM-TC-003</t>
+        </is>
+      </c>
+      <c r="D108" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E108" s="10" t="inlineStr">
+        <is>
+          <t>Product rule sets 200</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B109" s="10" t="inlineStr">
+        <is>
+          <t>Product Management &amp; Catalog</t>
+        </is>
+      </c>
+      <c r="C109" s="10" t="inlineStr">
+        <is>
+          <t>PM-TC-004</t>
+        </is>
+      </c>
+      <c r="D109" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E109" s="10" t="inlineStr">
+        <is>
+          <t>Product catalog views 200</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B110" s="10" t="inlineStr">
+        <is>
+          <t>Product Management &amp; Catalog</t>
+        </is>
+      </c>
+      <c r="C110" s="10" t="inlineStr">
+        <is>
+          <t>PM-TC-010</t>
+        </is>
+      </c>
+      <c r="D110" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E110" s="10" t="inlineStr">
+        <is>
+          <t>Create product family</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B111" s="10" t="inlineStr">
+        <is>
+          <t>Product Management &amp; Catalog</t>
+        </is>
+      </c>
+      <c r="C111" s="10" t="inlineStr">
+        <is>
+          <t>PM-TC-011</t>
+        </is>
+      </c>
+      <c r="D111" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E111" s="10" t="inlineStr">
+        <is>
+          <t>Create product category</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B112" s="10" t="inlineStr">
+        <is>
+          <t>Product Management &amp; Catalog</t>
+        </is>
+      </c>
+      <c r="C112" s="10" t="inlineStr">
+        <is>
+          <t>PM-TC-012</t>
+        </is>
+      </c>
+      <c r="D112" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E112" s="10" t="inlineStr">
+        <is>
+          <t>SALES_BD_REP denied catalog manage</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="10" t="inlineStr">
+        <is>
+          <t>WEB-UI</t>
+        </is>
+      </c>
+      <c r="B113" s="10" t="inlineStr">
+        <is>
+          <t>Product Management &amp; Catalog</t>
+        </is>
+      </c>
+      <c r="C113" s="10" t="inlineStr">
+        <is>
+          <t>Web page renders: /product-management</t>
+        </is>
+      </c>
+      <c r="D113" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E113" s="10" t="inlineStr">
+        <is>
+          <t>Rendered correctly; saw ["Product","Pulse"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B114" s="10" t="inlineStr">
+        <is>
+          <t>Reporting &amp; Dashboards</t>
+        </is>
+      </c>
+      <c r="C114" s="10" t="inlineStr">
+        <is>
+          <t>RPT-TC-001</t>
+        </is>
+      </c>
+      <c r="D114" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E114" s="10" t="inlineStr">
+        <is>
+          <t>Lead dashboard returns 200 for SUPER_ADMIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B115" s="10" t="inlineStr">
+        <is>
+          <t>Reporting &amp; Dashboards</t>
+        </is>
+      </c>
+      <c r="C115" s="10" t="inlineStr">
+        <is>
+          <t>RPT-TC-002</t>
+        </is>
+      </c>
+      <c r="D115" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E115" s="10" t="inlineStr">
+        <is>
+          <t>Training dashboard returns 200 for SUPER_ADMIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B116" s="10" t="inlineStr">
+        <is>
+          <t>Reporting &amp; Dashboards</t>
+        </is>
+      </c>
+      <c r="C116" s="10" t="inlineStr">
+        <is>
+          <t>RPT-TC-003</t>
+        </is>
+      </c>
+      <c r="D116" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E116" s="10" t="inlineStr">
+        <is>
+          <t>Executive dashboard returns 200 for SUPER_ADMIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B117" s="10" t="inlineStr">
+        <is>
+          <t>Reporting &amp; Dashboards</t>
+        </is>
+      </c>
+      <c r="C117" s="10" t="inlineStr">
+        <is>
+          <t>RPT-TC-020</t>
+        </is>
+      </c>
+      <c r="D117" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E117" s="10" t="inlineStr">
+        <is>
+          <t>EXECUTIVE can view executive dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B118" s="10" t="inlineStr">
+        <is>
+          <t>Reporting &amp; Dashboards</t>
+        </is>
+      </c>
+      <c r="C118" s="10" t="inlineStr">
+        <is>
+          <t>RPT-TC-021</t>
+        </is>
+      </c>
+      <c r="D118" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E118" s="10" t="inlineStr">
+        <is>
+          <t>TM denied executive dashboard (reports.executive gate)</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B119" s="10" t="inlineStr">
+        <is>
+          <t>Reporting &amp; Dashboards</t>
+        </is>
+      </c>
+      <c r="C119" s="10" t="inlineStr">
+        <is>
+          <t>RPT-TC-039</t>
+        </is>
+      </c>
+      <c r="D119" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E119" s="10" t="inlineStr">
+        <is>
+          <t>Stale/neglected accounts report 200</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B120" s="10" t="inlineStr">
+        <is>
+          <t>Reporting &amp; Dashboards</t>
+        </is>
+      </c>
+      <c r="C120" s="10" t="inlineStr">
+        <is>
+          <t>RPT-TC-003b</t>
+        </is>
+      </c>
+      <c r="D120" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E120" s="10" t="inlineStr">
+        <is>
+          <t>Threshold settings readable</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B121" s="10" t="inlineStr">
+        <is>
+          <t>Reporting &amp; Dashboards</t>
+        </is>
+      </c>
+      <c r="C121" s="10" t="inlineStr">
+        <is>
+          <t>RPT-TC-022b</t>
+        </is>
+      </c>
+      <c r="D121" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E121" s="10" t="inlineStr">
+        <is>
+          <t>TM threshold-settings access controlled (200)</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B122" s="10" t="inlineStr">
+        <is>
+          <t>Reporting &amp; Dashboards</t>
+        </is>
+      </c>
+      <c r="C122" s="10" t="inlineStr">
+        <is>
+          <t>RPT-TC-064</t>
+        </is>
+      </c>
+      <c r="D122" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E122" s="10" t="inlineStr">
+        <is>
+          <t>List report definitions</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B123" s="10" t="inlineStr">
+        <is>
+          <t>Reporting &amp; Dashboards</t>
+        </is>
+      </c>
+      <c r="C123" s="10" t="inlineStr">
+        <is>
+          <t>RPT-RUN-lead_funnel</t>
+        </is>
+      </c>
+      <c r="D123" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E123" s="10" t="inlineStr">
+        <is>
+          <t>Run ad-hoc report lead_funnel</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B124" s="10" t="inlineStr">
+        <is>
+          <t>Reporting &amp; Dashboards</t>
+        </is>
+      </c>
+      <c r="C124" s="10" t="inlineStr">
+        <is>
+          <t>RPT-RUN-training_compliance</t>
+        </is>
+      </c>
+      <c r="D124" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E124" s="10" t="inlineStr">
+        <is>
+          <t>Run ad-hoc report training_compliance</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B125" s="10" t="inlineStr">
+        <is>
+          <t>Reporting &amp; Dashboards</t>
+        </is>
+      </c>
+      <c r="C125" s="10" t="inlineStr">
+        <is>
+          <t>RPT-RUN-consignment_audit_status</t>
+        </is>
+      </c>
+      <c r="D125" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E125" s="10" t="inlineStr">
+        <is>
+          <t>Run ad-hoc report consignment_audit_status</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B126" s="10" t="inlineStr">
+        <is>
+          <t>Reporting &amp; Dashboards</t>
+        </is>
+      </c>
+      <c r="C126" s="10" t="inlineStr">
+        <is>
+          <t>RPT-RUN-field_activity</t>
+        </is>
+      </c>
+      <c r="D126" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E126" s="10" t="inlineStr">
+        <is>
+          <t>Run ad-hoc report field_activity</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="10" t="inlineStr">
+        <is>
+          <t>WEB-UI</t>
+        </is>
+      </c>
+      <c r="B127" s="10" t="inlineStr">
+        <is>
+          <t>Reporting &amp; Dashboards</t>
+        </is>
+      </c>
+      <c r="C127" s="10" t="inlineStr">
+        <is>
+          <t>Reports: dashboard Export control present (CSV/Excel/PDF)</t>
+        </is>
+      </c>
+      <c r="D127" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E127" s="10" t="inlineStr">
+        <is>
+          <t>Export button rendered on dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="10" t="inlineStr">
+        <is>
+          <t>WEB-UI</t>
+        </is>
+      </c>
+      <c r="B128" s="10" t="inlineStr">
+        <is>
+          <t>Reporting &amp; Dashboards</t>
+        </is>
+      </c>
+      <c r="C128" s="10" t="inlineStr">
+        <is>
+          <t>Web page renders: /reports</t>
+        </is>
+      </c>
+      <c r="D128" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E128" s="10" t="inlineStr">
+        <is>
+          <t>Rendered correctly; saw ["Reports","Export"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B129" s="10" t="inlineStr">
+        <is>
+          <t>Territory</t>
+        </is>
+      </c>
+      <c r="C129" s="10" t="inlineStr">
+        <is>
+          <t>TER-TC-001</t>
+        </is>
+      </c>
+      <c r="D129" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E129" s="10" t="inlineStr">
+        <is>
+          <t>Territory list 200</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B130" s="10" t="inlineStr">
+        <is>
+          <t>Territory</t>
+        </is>
+      </c>
+      <c r="C130" s="10" t="inlineStr">
+        <is>
+          <t>TER-TC-002</t>
+        </is>
+      </c>
+      <c r="D130" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E130" s="10" t="inlineStr">
+        <is>
+          <t>Territory regions 200</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B131" s="10" t="inlineStr">
+        <is>
+          <t>Territory</t>
+        </is>
+      </c>
+      <c r="C131" s="10" t="inlineStr">
+        <is>
+          <t>TER-TC-003</t>
+        </is>
+      </c>
+      <c r="D131" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E131" s="10" t="inlineStr">
+        <is>
+          <t>Territory map 200</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B132" s="10" t="inlineStr">
+        <is>
+          <t>Territory</t>
+        </is>
+      </c>
+      <c r="C132" s="10" t="inlineStr">
+        <is>
+          <t>TER-TC-004</t>
+        </is>
+      </c>
+      <c r="D132" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E132" s="10" t="inlineStr">
+        <is>
+          <t>Territory dashboard 200</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B133" s="10" t="inlineStr">
+        <is>
+          <t>Territory</t>
+        </is>
+      </c>
+      <c r="C133" s="10" t="inlineStr">
+        <is>
+          <t>TER-TC-010</t>
+        </is>
+      </c>
+      <c r="D133" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E133" s="10" t="inlineStr">
+        <is>
+          <t>TM can read territories</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B134" s="10" t="inlineStr">
+        <is>
+          <t>Territory</t>
+        </is>
+      </c>
+      <c r="C134" s="10" t="inlineStr">
+        <is>
+          <t>TER-TC-020</t>
+        </is>
+      </c>
+      <c r="D134" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E134" s="10" t="inlineStr">
+        <is>
+          <t>Territory assignable users</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B135" s="10" t="inlineStr">
+        <is>
+          <t>Territory</t>
+        </is>
+      </c>
+      <c r="C135" s="10" t="inlineStr">
+        <is>
+          <t>TER-TC-021</t>
+        </is>
+      </c>
+      <c r="D135" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E135" s="10" t="inlineStr">
+        <is>
+          <t>Territory policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B136" s="10" t="inlineStr">
+        <is>
+          <t>Territory</t>
+        </is>
+      </c>
+      <c r="C136" s="10" t="inlineStr">
+        <is>
+          <t>TER-TC-023</t>
+        </is>
+      </c>
+      <c r="D136" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E136" s="10" t="inlineStr">
+        <is>
+          <t>Territory shipping centers</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="10" t="inlineStr">
+        <is>
+          <t>WEB-UI</t>
+        </is>
+      </c>
+      <c r="B137" s="10" t="inlineStr">
+        <is>
+          <t>Territory</t>
+        </is>
+      </c>
+      <c r="C137" s="10" t="inlineStr">
+        <is>
+          <t>Web page renders: /territories</t>
+        </is>
+      </c>
+      <c r="D137" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E137" s="10" t="inlineStr">
+        <is>
+          <t>Rendered correctly; saw ["Territor","Pulse"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="10" t="inlineStr">
+        <is>
+          <t>WEB-UI</t>
+        </is>
+      </c>
+      <c r="B138" s="10" t="inlineStr">
+        <is>
+          <t>Territory</t>
+        </is>
+      </c>
+      <c r="C138" s="10" t="inlineStr">
+        <is>
+          <t>Web page renders: /territory_map</t>
+        </is>
+      </c>
+      <c r="D138" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E138" s="10" t="inlineStr">
+        <is>
+          <t>Rendered correctly; saw ["Pulse"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B139" s="10" t="inlineStr">
         <is>
           <t>Training</t>
         </is>
       </c>
-      <c r="C100" s="10" t="inlineStr">
+      <c r="C139" s="10" t="inlineStr">
+        <is>
+          <t>TRN-TC-001</t>
+        </is>
+      </c>
+      <c r="D139" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E139" s="10" t="inlineStr">
+        <is>
+          <t>Training sessions 200</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B140" s="10" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="C140" s="10" t="inlineStr">
+        <is>
+          <t>TRN-TC-002</t>
+        </is>
+      </c>
+      <c r="D140" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E140" s="10" t="inlineStr">
+        <is>
+          <t>Training overview 200</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B141" s="10" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="C141" s="10" t="inlineStr">
+        <is>
+          <t>TRN-TC-003</t>
+        </is>
+      </c>
+      <c r="D141" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E141" s="10" t="inlineStr">
+        <is>
+          <t>Training catalog 200</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B142" s="10" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="C142" s="10" t="inlineStr">
+        <is>
+          <t>TRN-TC-004</t>
+        </is>
+      </c>
+      <c r="D142" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E142" s="10" t="inlineStr">
+        <is>
+          <t>Training trainers 200</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B143" s="10" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="C143" s="10" t="inlineStr">
+        <is>
+          <t>TRN-TC-010</t>
+        </is>
+      </c>
+      <c r="D143" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E143" s="10" t="inlineStr">
+        <is>
+          <t>TRAINING_OPS can read sessions</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B144" s="10" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="C144" s="10" t="inlineStr">
+        <is>
+          <t>TRN-TC-020</t>
+        </is>
+      </c>
+      <c r="D144" s="14" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="E144" s="10" t="inlineStr">
+        <is>
+          <t>schedule session -&gt; 400: Training type not found</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B145" s="10" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="C145" s="10" t="inlineStr">
+        <is>
+          <t>TRN-TC-023</t>
+        </is>
+      </c>
+      <c r="D145" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E145" s="10" t="inlineStr">
+        <is>
+          <t>FINANCE denied training.schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="10" t="inlineStr">
+        <is>
+          <t>WEB-UI</t>
+        </is>
+      </c>
+      <c r="B146" s="10" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="C146" s="10" t="inlineStr">
         <is>
           <t>Web page renders: /training</t>
         </is>
       </c>
-      <c r="D100" s="13" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="E100" s="10" t="inlineStr">
+      <c r="D146" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E146" s="10" t="inlineStr">
         <is>
           <t>Rendered correctly; saw ["Training","Pulse"]</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:E100"/>
+  <autoFilter ref="A3:E146"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(qa): add Dealer Portal ordering + Mobile voice-note execution (214 live checks, 207 PASS)
Reset a seeded dealer login and executed the full dealer ordering flow (auth -> catalog -> add-to-cart -> submit
with PO number -> portal isolation both directions) and the mobile voice-notes API (create at /mobile/voice-notes,
PCI rejection of a PAN in a transcript, review-queue, list, reviewer approve). All 18 PASS. Verified order-submit
correctly requires a PO number and dealer<->internal isolation holds. Live now 214 checks (UI 21 + API 193):
207 PASS, 1 FAIL (consignment PCI gap, in-branch fix 327b6e9 not deployed), 6 PARTIAL.

Co-Authored-By: claude-flow <ruv@ruv.net>
</commit_message>
<xml_diff>
--- a/docs/test-plan/Pulse_CRM_Module_Execution_Report.xlsx
+++ b/docs/test-plan/Pulse_CRM_Module_Execution_Report.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'GAPS (FAILED)'!$A$4:$F$132</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Executed (live)'!$A$3:$E$199</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Executed (live)'!$A$3:$E$217</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -788,8 +788,8 @@
       <c r="B12" s="5" t="n">
         <v>68</v>
       </c>
-      <c r="C12" s="5" t="n">
-        <v>0</v>
+      <c r="C12" s="6" t="n">
+        <v>5</v>
       </c>
       <c r="D12" s="5" t="n">
         <v>0</v>
@@ -798,7 +798,7 @@
         <v>7</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
@@ -897,7 +897,7 @@
         <v>56</v>
       </c>
       <c r="C16" s="6" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="D16" s="5" t="n">
         <v>0</v>
@@ -906,7 +906,7 @@
         <v>14</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
@@ -1086,7 +1086,7 @@
         <v>1047</v>
       </c>
       <c r="C23" s="8" t="n">
-        <v>189</v>
+        <v>207</v>
       </c>
       <c r="D23" s="8" t="n">
         <v>1</v>
@@ -1095,7 +1095,7 @@
         <v>128</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>723</v>
+        <v>705</v>
       </c>
       <c r="G23" s="8" t="inlineStr"/>
     </row>
@@ -5275,7 +5275,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E199"/>
+  <dimension ref="A1:E217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5288,7 +5288,7 @@
     <row r="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
-          <t>Live-executed checks — Web UI (21) + API (175)</t>
+          <t>Live-executed checks — Web UI (21) + API (193)</t>
         </is>
       </c>
     </row>
@@ -7266,7 +7266,7 @@
     <row r="76">
       <c r="A76" s="10" t="inlineStr">
         <is>
-          <t>WEB-UI</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B76" s="10" t="inlineStr">
@@ -7276,7 +7276,7 @@
       </c>
       <c r="C76" s="10" t="inlineStr">
         <is>
-          <t>Web page renders: /dealer/login</t>
+          <t>DLR-TC-010</t>
         </is>
       </c>
       <c r="D76" s="13" t="inlineStr">
@@ -7286,7 +7286,7 @@
       </c>
       <c r="E76" s="10" t="inlineStr">
         <is>
-          <t>Rendered correctly; saw ["Dealer","Sign"]</t>
+          <t>Dealer (DEALER_PORTAL_USER) can authenticate</t>
         </is>
       </c>
     </row>
@@ -7298,12 +7298,12 @@
       </c>
       <c r="B77" s="10" t="inlineStr">
         <is>
-          <t>Digital Assets (DAM)</t>
+          <t>Dealer Portal &amp; Ordering</t>
         </is>
       </c>
       <c r="C77" s="10" t="inlineStr">
         <is>
-          <t>DAM-TC-001</t>
+          <t>DLR-TC-011</t>
         </is>
       </c>
       <c r="D77" s="13" t="inlineStr">
@@ -7313,7 +7313,7 @@
       </c>
       <c r="E77" s="10" t="inlineStr">
         <is>
-          <t>DAM assets 200</t>
+          <t>Dealer dashboard loads</t>
         </is>
       </c>
     </row>
@@ -7325,12 +7325,12 @@
       </c>
       <c r="B78" s="10" t="inlineStr">
         <is>
-          <t>Digital Assets (DAM)</t>
+          <t>Dealer Portal &amp; Ordering</t>
         </is>
       </c>
       <c r="C78" s="10" t="inlineStr">
         <is>
-          <t>DAM-TC-002</t>
+          <t>DLR-TC-012</t>
         </is>
       </c>
       <c r="D78" s="13" t="inlineStr">
@@ -7340,7 +7340,7 @@
       </c>
       <c r="E78" s="10" t="inlineStr">
         <is>
-          <t>DAM collections 200</t>
+          <t>Dealer catalog loads</t>
         </is>
       </c>
     </row>
@@ -7352,12 +7352,12 @@
       </c>
       <c r="B79" s="10" t="inlineStr">
         <is>
-          <t>Digital Assets (DAM)</t>
+          <t>Dealer Portal &amp; Ordering</t>
         </is>
       </c>
       <c r="C79" s="10" t="inlineStr">
         <is>
-          <t>DAM-TC-011</t>
+          <t>DLR-TC-013</t>
         </is>
       </c>
       <c r="D79" s="13" t="inlineStr">
@@ -7367,7 +7367,7 @@
       </c>
       <c r="E79" s="10" t="inlineStr">
         <is>
-          <t>DAM Widen import runs list</t>
+          <t>Dealer cart loads</t>
         </is>
       </c>
     </row>
@@ -7379,12 +7379,12 @@
       </c>
       <c r="B80" s="10" t="inlineStr">
         <is>
-          <t>Digital Assets (DAM)</t>
+          <t>Dealer Portal &amp; Ordering</t>
         </is>
       </c>
       <c r="C80" s="10" t="inlineStr">
         <is>
-          <t>DAM-TC-012</t>
+          <t>DLR-TC-014</t>
         </is>
       </c>
       <c r="D80" s="13" t="inlineStr">
@@ -7394,7 +7394,7 @@
       </c>
       <c r="E80" s="10" t="inlineStr">
         <is>
-          <t>DAM Widen import preview endpoint reachable (405)</t>
+          <t>Dealer orders loads</t>
         </is>
       </c>
     </row>
@@ -7406,12 +7406,12 @@
       </c>
       <c r="B81" s="10" t="inlineStr">
         <is>
-          <t>Digital Assets (DAM)</t>
+          <t>Dealer Portal &amp; Ordering</t>
         </is>
       </c>
       <c r="C81" s="10" t="inlineStr">
         <is>
-          <t>DAM-READ-23</t>
+          <t>DLR-TC-015</t>
         </is>
       </c>
       <c r="D81" s="13" t="inlineStr">
@@ -7421,7 +7421,7 @@
       </c>
       <c r="E81" s="10" t="inlineStr">
         <is>
-          <t>GET /digital-assets/assets -&gt; 200 (loads/lists for authorised user)</t>
+          <t>Dealer adds product to cart</t>
         </is>
       </c>
     </row>
@@ -7433,12 +7433,12 @@
       </c>
       <c r="B82" s="10" t="inlineStr">
         <is>
-          <t>Digital Assets (DAM)</t>
+          <t>Dealer Portal &amp; Ordering</t>
         </is>
       </c>
       <c r="C82" s="10" t="inlineStr">
         <is>
-          <t>DAM-READ-24</t>
+          <t>DLR-TC-016</t>
         </is>
       </c>
       <c r="D82" s="13" t="inlineStr">
@@ -7448,7 +7448,7 @@
       </c>
       <c r="E82" s="10" t="inlineStr">
         <is>
-          <t>GET /digital-assets/collections -&gt; 200 (loads/lists for authorised user)</t>
+          <t>Cart reflects added items (1)</t>
         </is>
       </c>
     </row>
@@ -7460,12 +7460,12 @@
       </c>
       <c r="B83" s="10" t="inlineStr">
         <is>
-          <t>Digital Assets (DAM)</t>
+          <t>Dealer Portal &amp; Ordering</t>
         </is>
       </c>
       <c r="C83" s="10" t="inlineStr">
         <is>
-          <t>DAM-READ-25</t>
+          <t>DLR-TC-017</t>
         </is>
       </c>
       <c r="D83" s="13" t="inlineStr">
@@ -7475,24 +7475,24 @@
       </c>
       <c r="E83" s="10" t="inlineStr">
         <is>
-          <t>GET /digital-assets/widen-import-runs -&gt; 200 (loads/lists for authorised user)</t>
+          <t>Dealer submits order</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="10" t="inlineStr">
         <is>
-          <t>WEB-UI</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B84" s="10" t="inlineStr">
         <is>
-          <t>Digital Assets (DAM)</t>
+          <t>Dealer Portal &amp; Ordering</t>
         </is>
       </c>
       <c r="C84" s="10" t="inlineStr">
         <is>
-          <t>Web page renders: /digital-assets</t>
+          <t>DLR-TC-018</t>
         </is>
       </c>
       <c r="D84" s="13" t="inlineStr">
@@ -7502,24 +7502,24 @@
       </c>
       <c r="E84" s="10" t="inlineStr">
         <is>
-          <t>Rendered correctly; saw ["Digital Assets","Library"]</t>
+          <t>Dealer correctly blocked from internal /leads</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="10" t="inlineStr">
         <is>
-          <t>WEB-UI</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B85" s="10" t="inlineStr">
         <is>
-          <t>Digital Assets (DAM)</t>
+          <t>Dealer Portal &amp; Ordering</t>
         </is>
       </c>
       <c r="C85" s="10" t="inlineStr">
         <is>
-          <t>Web page renders: /digital-assets?tab=migration</t>
+          <t>DLR-TC-019</t>
         </is>
       </c>
       <c r="D85" s="13" t="inlineStr">
@@ -7529,7 +7529,7 @@
       </c>
       <c r="E85" s="10" t="inlineStr">
         <is>
-          <t>Rendered correctly; saw ["Migration Review","Widen"]</t>
+          <t>Dealer correctly blocked from internal /admin/users</t>
         </is>
       </c>
     </row>
@@ -7541,12 +7541,12 @@
       </c>
       <c r="B86" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Dealer Portal &amp; Ordering</t>
         </is>
       </c>
       <c r="C86" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-005</t>
+          <t>DLR-TC-020</t>
         </is>
       </c>
       <c r="D86" s="13" t="inlineStr">
@@ -7556,7 +7556,7 @@
       </c>
       <c r="E86" s="10" t="inlineStr">
         <is>
-          <t>Authorized user created a manual lead</t>
+          <t>Dealer correctly blocked from internal /accounts</t>
         </is>
       </c>
     </row>
@@ -7568,12 +7568,12 @@
       </c>
       <c r="B87" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Dealer Portal &amp; Ordering</t>
         </is>
       </c>
       <c r="C87" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-006a</t>
+          <t>DLR-TC-021</t>
         </is>
       </c>
       <c r="D87" s="13" t="inlineStr">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="E87" s="10" t="inlineStr">
         <is>
-          <t>TERRITORY_MANAGER correctly denied lead creation (default-deny)</t>
+          <t>TERRITORY_MANAGER has no dealer /me context (403)</t>
         </is>
       </c>
     </row>
@@ -7595,12 +7595,12 @@
       </c>
       <c r="B88" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Dealer Portal &amp; Ordering</t>
         </is>
       </c>
       <c r="C88" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-006b</t>
+          <t>DLR-TC-022</t>
         </is>
       </c>
       <c r="D88" s="13" t="inlineStr">
@@ -7610,24 +7610,24 @@
       </c>
       <c r="E88" s="10" t="inlineStr">
         <is>
-          <t>REGIONAL_DIRECTOR correctly denied lead creation (default-deny)</t>
+          <t>SALES_BD_REP has no dealer /me context (403)</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="10" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>WEB-UI</t>
         </is>
       </c>
       <c r="B89" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Dealer Portal &amp; Ordering</t>
         </is>
       </c>
       <c r="C89" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-006c</t>
+          <t>Web page renders: /dealer/login</t>
         </is>
       </c>
       <c r="D89" s="13" t="inlineStr">
@@ -7637,7 +7637,7 @@
       </c>
       <c r="E89" s="10" t="inlineStr">
         <is>
-          <t>FINANCE correctly denied lead creation (default-deny)</t>
+          <t>Rendered correctly; saw ["Dealer","Sign"]</t>
         </is>
       </c>
     </row>
@@ -7649,12 +7649,12 @@
       </c>
       <c r="B90" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Digital Assets (DAM)</t>
         </is>
       </c>
       <c r="C90" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-007</t>
+          <t>DAM-TC-001</t>
         </is>
       </c>
       <c r="D90" s="13" t="inlineStr">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="E90" s="10" t="inlineStr">
         <is>
-          <t>Invalid email rejected at intake</t>
+          <t>DAM assets 200</t>
         </is>
       </c>
     </row>
@@ -7676,12 +7676,12 @@
       </c>
       <c r="B91" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Digital Assets (DAM)</t>
         </is>
       </c>
       <c r="C91" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-008</t>
+          <t>DAM-TC-002</t>
         </is>
       </c>
       <c r="D91" s="13" t="inlineStr">
@@ -7691,7 +7691,7 @@
       </c>
       <c r="E91" s="10" t="inlineStr">
         <is>
-          <t>Invalid phone (too few digits) rejected</t>
+          <t>DAM collections 200</t>
         </is>
       </c>
     </row>
@@ -7703,12 +7703,12 @@
       </c>
       <c r="B92" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Digital Assets (DAM)</t>
         </is>
       </c>
       <c r="C92" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-009</t>
+          <t>DAM-TC-011</t>
         </is>
       </c>
       <c r="D92" s="13" t="inlineStr">
@@ -7718,7 +7718,7 @@
       </c>
       <c r="E92" s="10" t="inlineStr">
         <is>
-          <t>Missing company rejected</t>
+          <t>DAM Widen import runs list</t>
         </is>
       </c>
     </row>
@@ -7730,12 +7730,12 @@
       </c>
       <c r="B93" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Digital Assets (DAM)</t>
         </is>
       </c>
       <c r="C93" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-031</t>
+          <t>DAM-TC-012</t>
         </is>
       </c>
       <c r="D93" s="13" t="inlineStr">
@@ -7745,7 +7745,7 @@
       </c>
       <c r="E93" s="10" t="inlineStr">
         <is>
-          <t>PCI: raw card number in lead note rejected</t>
+          <t>DAM Widen import preview endpoint reachable (405)</t>
         </is>
       </c>
     </row>
@@ -7757,12 +7757,12 @@
       </c>
       <c r="B94" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Digital Assets (DAM)</t>
         </is>
       </c>
       <c r="C94" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-040</t>
+          <t>DAM-READ-23</t>
         </is>
       </c>
       <c r="D94" s="13" t="inlineStr">
@@ -7772,7 +7772,7 @@
       </c>
       <c r="E94" s="10" t="inlineStr">
         <is>
-          <t>Lead list returns items</t>
+          <t>GET /digital-assets/assets -&gt; 200 (loads/lists for authorised user)</t>
         </is>
       </c>
     </row>
@@ -7784,12 +7784,12 @@
       </c>
       <c r="B95" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Digital Assets (DAM)</t>
         </is>
       </c>
       <c r="C95" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-041</t>
+          <t>DAM-READ-24</t>
         </is>
       </c>
       <c r="D95" s="13" t="inlineStr">
@@ -7799,7 +7799,7 @@
       </c>
       <c r="E95" s="10" t="inlineStr">
         <is>
-          <t>Non-existent lead returns not-found/forbidden</t>
+          <t>GET /digital-assets/collections -&gt; 200 (loads/lists for authorised user)</t>
         </is>
       </c>
     </row>
@@ -7811,12 +7811,12 @@
       </c>
       <c r="B96" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Digital Assets (DAM)</t>
         </is>
       </c>
       <c r="C96" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-053</t>
+          <t>DAM-READ-25</t>
         </is>
       </c>
       <c r="D96" s="13" t="inlineStr">
@@ -7826,24 +7826,24 @@
       </c>
       <c r="E96" s="10" t="inlineStr">
         <is>
-          <t>Duplicate detection: 2nd lead with same phone is blocked pending resolution (400)</t>
+          <t>GET /digital-assets/widen-import-runs -&gt; 200 (loads/lists for authorised user)</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>WEB-UI</t>
         </is>
       </c>
       <c r="B97" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Digital Assets (DAM)</t>
         </is>
       </c>
       <c r="C97" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-008b</t>
+          <t>Web page renders: /digital-assets</t>
         </is>
       </c>
       <c r="D97" s="13" t="inlineStr">
@@ -7853,24 +7853,24 @@
       </c>
       <c r="E97" s="10" t="inlineStr">
         <is>
-          <t>7-digit phone (lower boundary) accepted</t>
+          <t>Rendered correctly; saw ["Digital Assets","Library"]</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="10" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>WEB-UI</t>
         </is>
       </c>
       <c r="B98" s="10" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Digital Assets (DAM)</t>
         </is>
       </c>
       <c r="C98" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-008c</t>
+          <t>Web page renders: /digital-assets?tab=migration</t>
         </is>
       </c>
       <c r="D98" s="13" t="inlineStr">
@@ -7880,7 +7880,7 @@
       </c>
       <c r="E98" s="10" t="inlineStr">
         <is>
-          <t>16-digit phone (over boundary) rejected</t>
+          <t>Rendered correctly; saw ["Migration Review","Widen"]</t>
         </is>
       </c>
     </row>
@@ -7897,7 +7897,7 @@
       </c>
       <c r="C99" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-050</t>
+          <t>LEAD-TC-005</t>
         </is>
       </c>
       <c r="D99" s="13" t="inlineStr">
@@ -7907,7 +7907,7 @@
       </c>
       <c r="E99" s="10" t="inlineStr">
         <is>
-          <t>Special chars / SQL-ish input handled without server error</t>
+          <t>Authorized user created a manual lead</t>
         </is>
       </c>
     </row>
@@ -7924,7 +7924,7 @@
       </c>
       <c r="C100" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-051</t>
+          <t>LEAD-TC-006a</t>
         </is>
       </c>
       <c r="D100" s="13" t="inlineStr">
@@ -7934,7 +7934,7 @@
       </c>
       <c r="E100" s="10" t="inlineStr">
         <is>
-          <t>Oversized field handled gracefully (400)</t>
+          <t>TERRITORY_MANAGER correctly denied lead creation (default-deny)</t>
         </is>
       </c>
     </row>
@@ -7951,7 +7951,7 @@
       </c>
       <c r="C101" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-052</t>
+          <t>LEAD-TC-006b</t>
         </is>
       </c>
       <c r="D101" s="13" t="inlineStr">
@@ -7961,7 +7961,7 @@
       </c>
       <c r="E101" s="10" t="inlineStr">
         <is>
-          <t>Pagination limit honoured (&lt;=2 items)</t>
+          <t>REGIONAL_DIRECTOR correctly denied lead creation (default-deny)</t>
         </is>
       </c>
     </row>
@@ -7978,7 +7978,7 @@
       </c>
       <c r="C102" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-020</t>
+          <t>LEAD-TC-006c</t>
         </is>
       </c>
       <c r="D102" s="13" t="inlineStr">
@@ -7988,7 +7988,7 @@
       </c>
       <c r="E102" s="10" t="inlineStr">
         <is>
-          <t>Discovery scheduled</t>
+          <t>FINANCE correctly denied lead creation (default-deny)</t>
         </is>
       </c>
     </row>
@@ -8005,7 +8005,7 @@
       </c>
       <c r="C103" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-021</t>
+          <t>LEAD-TC-007</t>
         </is>
       </c>
       <c r="D103" s="13" t="inlineStr">
@@ -8015,7 +8015,7 @@
       </c>
       <c r="E103" s="10" t="inlineStr">
         <is>
-          <t>Discovery completed (lead advanced)</t>
+          <t>Invalid email rejected at intake</t>
         </is>
       </c>
     </row>
@@ -8032,7 +8032,7 @@
       </c>
       <c r="C104" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-002b</t>
+          <t>LEAD-TC-008</t>
         </is>
       </c>
       <c r="D104" s="13" t="inlineStr">
@@ -8042,7 +8042,7 @@
       </c>
       <c r="E104" s="10" t="inlineStr">
         <is>
-          <t>Create lead (deep fixture)</t>
+          <t>Invalid phone (too few digits) rejected</t>
         </is>
       </c>
     </row>
@@ -8059,7 +8059,7 @@
       </c>
       <c r="C105" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-060</t>
+          <t>LEAD-TC-009</t>
         </is>
       </c>
       <c r="D105" s="13" t="inlineStr">
@@ -8069,7 +8069,7 @@
       </c>
       <c r="E105" s="10" t="inlineStr">
         <is>
-          <t>Add lead contact</t>
+          <t>Missing company rejected</t>
         </is>
       </c>
     </row>
@@ -8086,7 +8086,7 @@
       </c>
       <c r="C106" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-061</t>
+          <t>LEAD-TC-031</t>
         </is>
       </c>
       <c r="D106" s="13" t="inlineStr">
@@ -8096,7 +8096,7 @@
       </c>
       <c r="E106" s="10" t="inlineStr">
         <is>
-          <t>List lead contacts</t>
+          <t>PCI: raw card number in lead note rejected</t>
         </is>
       </c>
     </row>
@@ -8113,7 +8113,7 @@
       </c>
       <c r="C107" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-062</t>
+          <t>LEAD-TC-040</t>
         </is>
       </c>
       <c r="D107" s="13" t="inlineStr">
@@ -8123,7 +8123,7 @@
       </c>
       <c r="E107" s="10" t="inlineStr">
         <is>
-          <t>Log activity note</t>
+          <t>Lead list returns items</t>
         </is>
       </c>
     </row>
@@ -8140,7 +8140,7 @@
       </c>
       <c r="C108" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-070</t>
+          <t>LEAD-TC-041</t>
         </is>
       </c>
       <c r="D108" s="13" t="inlineStr">
@@ -8150,7 +8150,7 @@
       </c>
       <c r="E108" s="10" t="inlineStr">
         <is>
-          <t>Lead readiness loads</t>
+          <t>Non-existent lead returns not-found/forbidden</t>
         </is>
       </c>
     </row>
@@ -8167,7 +8167,7 @@
       </c>
       <c r="C109" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-072</t>
+          <t>LEAD-TC-053</t>
         </is>
       </c>
       <c r="D109" s="13" t="inlineStr">
@@ -8177,7 +8177,7 @@
       </c>
       <c r="E109" s="10" t="inlineStr">
         <is>
-          <t>Lead readiness blockers loads</t>
+          <t>Duplicate detection: 2nd lead with same phone is blocked pending resolution (400)</t>
         </is>
       </c>
     </row>
@@ -8194,7 +8194,7 @@
       </c>
       <c r="C110" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-073</t>
+          <t>LEAD-TC-008b</t>
         </is>
       </c>
       <c r="D110" s="13" t="inlineStr">
@@ -8204,7 +8204,7 @@
       </c>
       <c r="E110" s="10" t="inlineStr">
         <is>
-          <t>Log initial contact</t>
+          <t>7-digit phone (lower boundary) accepted</t>
         </is>
       </c>
     </row>
@@ -8221,7 +8221,7 @@
       </c>
       <c r="C111" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-074</t>
+          <t>LEAD-TC-008c</t>
         </is>
       </c>
       <c r="D111" s="13" t="inlineStr">
@@ -8231,7 +8231,7 @@
       </c>
       <c r="E111" s="10" t="inlineStr">
         <is>
-          <t>Lead search filter</t>
+          <t>16-digit phone (over boundary) rejected</t>
         </is>
       </c>
     </row>
@@ -8248,7 +8248,7 @@
       </c>
       <c r="C112" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-075</t>
+          <t>LEAD-TC-050</t>
         </is>
       </c>
       <c r="D112" s="13" t="inlineStr">
@@ -8258,7 +8258,7 @@
       </c>
       <c r="E112" s="10" t="inlineStr">
         <is>
-          <t>Lead stage filter</t>
+          <t>Special chars / SQL-ish input handled without server error</t>
         </is>
       </c>
     </row>
@@ -8275,7 +8275,7 @@
       </c>
       <c r="C113" s="10" t="inlineStr">
         <is>
-          <t>LEAD-TC-076</t>
+          <t>LEAD-TC-051</t>
         </is>
       </c>
       <c r="D113" s="13" t="inlineStr">
@@ -8285,7 +8285,7 @@
       </c>
       <c r="E113" s="10" t="inlineStr">
         <is>
-          <t>TM can view leads (scoped)</t>
+          <t>Oversized field handled gracefully (400)</t>
         </is>
       </c>
     </row>
@@ -8302,7 +8302,7 @@
       </c>
       <c r="C114" s="10" t="inlineStr">
         <is>
-          <t>LEAD-READ-36</t>
+          <t>LEAD-TC-052</t>
         </is>
       </c>
       <c r="D114" s="13" t="inlineStr">
@@ -8312,7 +8312,7 @@
       </c>
       <c r="E114" s="10" t="inlineStr">
         <is>
-          <t>GET /leads -&gt; 200 (loads/lists for authorised user)</t>
+          <t>Pagination limit honoured (&lt;=2 items)</t>
         </is>
       </c>
     </row>
@@ -8329,7 +8329,7 @@
       </c>
       <c r="C115" s="10" t="inlineStr">
         <is>
-          <t>LEAD-RBAC-create_lead_(intak</t>
+          <t>LEAD-TC-020</t>
         </is>
       </c>
       <c r="D115" s="13" t="inlineStr">
@@ -8339,14 +8339,14 @@
       </c>
       <c r="E115" s="10" t="inlineStr">
         <is>
-          <t>Default-deny on "create lead (intake)": all 5 unauthorised roles got 403</t>
+          <t>Discovery scheduled</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="10" t="inlineStr">
         <is>
-          <t>WEB-UI</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B116" s="10" t="inlineStr">
@@ -8356,7 +8356,7 @@
       </c>
       <c r="C116" s="10" t="inlineStr">
         <is>
-          <t>Leads: list renders rows</t>
+          <t>LEAD-TC-021</t>
         </is>
       </c>
       <c r="D116" s="13" t="inlineStr">
@@ -8366,14 +8366,14 @@
       </c>
       <c r="E116" s="10" t="inlineStr">
         <is>
-          <t>104 lead rows/links present</t>
+          <t>Discovery completed (lead advanced)</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="10" t="inlineStr">
         <is>
-          <t>WEB-UI</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B117" s="10" t="inlineStr">
@@ -8383,7 +8383,7 @@
       </c>
       <c r="C117" s="10" t="inlineStr">
         <is>
-          <t>Web page renders: /leads</t>
+          <t>LEAD-TC-002b</t>
         </is>
       </c>
       <c r="D117" s="13" t="inlineStr">
@@ -8393,7 +8393,7 @@
       </c>
       <c r="E117" s="10" t="inlineStr">
         <is>
-          <t>Rendered correctly; saw ["Lead","QA-HVAC"]</t>
+          <t>Create lead (deep fixture)</t>
         </is>
       </c>
     </row>
@@ -8405,12 +8405,12 @@
       </c>
       <c r="B118" s="10" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C118" s="10" t="inlineStr">
         <is>
-          <t>NOT-TC-001</t>
+          <t>LEAD-TC-060</t>
         </is>
       </c>
       <c r="D118" s="13" t="inlineStr">
@@ -8420,7 +8420,7 @@
       </c>
       <c r="E118" s="10" t="inlineStr">
         <is>
-          <t>Notifications inbox list 200</t>
+          <t>Add lead contact</t>
         </is>
       </c>
     </row>
@@ -8432,12 +8432,12 @@
       </c>
       <c r="B119" s="10" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C119" s="10" t="inlineStr">
         <is>
-          <t>NOT-TC-002</t>
+          <t>LEAD-TC-061</t>
         </is>
       </c>
       <c r="D119" s="13" t="inlineStr">
@@ -8447,7 +8447,7 @@
       </c>
       <c r="E119" s="10" t="inlineStr">
         <is>
-          <t>Notifications unread count 200</t>
+          <t>List lead contacts</t>
         </is>
       </c>
     </row>
@@ -8459,12 +8459,12 @@
       </c>
       <c r="B120" s="10" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C120" s="10" t="inlineStr">
         <is>
-          <t>NOT-TC-003</t>
+          <t>LEAD-TC-062</t>
         </is>
       </c>
       <c r="D120" s="13" t="inlineStr">
@@ -8474,7 +8474,7 @@
       </c>
       <c r="E120" s="10" t="inlineStr">
         <is>
-          <t>Notifications preferences 200</t>
+          <t>Log activity note</t>
         </is>
       </c>
     </row>
@@ -8486,12 +8486,12 @@
       </c>
       <c r="B121" s="10" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C121" s="10" t="inlineStr">
         <is>
-          <t>NOT-TC-010</t>
+          <t>LEAD-TC-070</t>
         </is>
       </c>
       <c r="D121" s="13" t="inlineStr">
@@ -8501,7 +8501,7 @@
       </c>
       <c r="E121" s="10" t="inlineStr">
         <is>
-          <t>Admin can read routing rules</t>
+          <t>Lead readiness loads</t>
         </is>
       </c>
     </row>
@@ -8513,12 +8513,12 @@
       </c>
       <c r="B122" s="10" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C122" s="10" t="inlineStr">
         <is>
-          <t>NOT-TC-011</t>
+          <t>LEAD-TC-072</t>
         </is>
       </c>
       <c r="D122" s="13" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="E122" s="10" t="inlineStr">
         <is>
-          <t>Routing rules access for TM controlled (403)</t>
+          <t>Lead readiness blockers loads</t>
         </is>
       </c>
     </row>
@@ -8540,12 +8540,12 @@
       </c>
       <c r="B123" s="10" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C123" s="10" t="inlineStr">
         <is>
-          <t>NOT-TC-020</t>
+          <t>LEAD-TC-073</t>
         </is>
       </c>
       <c r="D123" s="13" t="inlineStr">
@@ -8555,7 +8555,7 @@
       </c>
       <c r="E123" s="10" t="inlineStr">
         <is>
-          <t>Mark notifications read</t>
+          <t>Log initial contact</t>
         </is>
       </c>
     </row>
@@ -8567,22 +8567,22 @@
       </c>
       <c r="B124" s="10" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C124" s="10" t="inlineStr">
         <is>
-          <t>NOT-TC-021</t>
-        </is>
-      </c>
-      <c r="D124" s="14" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+          <t>LEAD-TC-074</t>
+        </is>
+      </c>
+      <c r="D124" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="E124" s="10" t="inlineStr">
         <is>
-          <t>400: A valid notification category is required.</t>
+          <t>Lead search filter</t>
         </is>
       </c>
     </row>
@@ -8594,12 +8594,12 @@
       </c>
       <c r="B125" s="10" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C125" s="10" t="inlineStr">
         <is>
-          <t>NOT-TC-022</t>
+          <t>LEAD-TC-075</t>
         </is>
       </c>
       <c r="D125" s="13" t="inlineStr">
@@ -8609,7 +8609,7 @@
       </c>
       <c r="E125" s="10" t="inlineStr">
         <is>
-          <t>Create notification routing rule</t>
+          <t>Lead stage filter</t>
         </is>
       </c>
     </row>
@@ -8621,12 +8621,12 @@
       </c>
       <c r="B126" s="10" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C126" s="10" t="inlineStr">
         <is>
-          <t>NOT-TC-023</t>
+          <t>LEAD-TC-076</t>
         </is>
       </c>
       <c r="D126" s="13" t="inlineStr">
@@ -8636,7 +8636,7 @@
       </c>
       <c r="E126" s="10" t="inlineStr">
         <is>
-          <t>Delete routing rule</t>
+          <t>TM can view leads (scoped)</t>
         </is>
       </c>
     </row>
@@ -8648,12 +8648,12 @@
       </c>
       <c r="B127" s="10" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C127" s="10" t="inlineStr">
         <is>
-          <t>NOT-TC-024</t>
+          <t>LEAD-READ-36</t>
         </is>
       </c>
       <c r="D127" s="13" t="inlineStr">
@@ -8663,7 +8663,7 @@
       </c>
       <c r="E127" s="10" t="inlineStr">
         <is>
-          <t>TM denied routing-rule creation (admin-gated)</t>
+          <t>GET /leads -&gt; 200 (loads/lists for authorised user)</t>
         </is>
       </c>
     </row>
@@ -8675,12 +8675,12 @@
       </c>
       <c r="B128" s="10" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C128" s="10" t="inlineStr">
         <is>
-          <t>NOT-READ-16</t>
+          <t>LEAD-RBAC-create_lead_(intak</t>
         </is>
       </c>
       <c r="D128" s="13" t="inlineStr">
@@ -8690,24 +8690,24 @@
       </c>
       <c r="E128" s="10" t="inlineStr">
         <is>
-          <t>GET /notifications/unread-count -&gt; 200 (loads/lists for authorised user)</t>
+          <t>Default-deny on "create lead (intake)": all 5 unauthorised roles got 403</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="10" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>WEB-UI</t>
         </is>
       </c>
       <c r="B129" s="10" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C129" s="10" t="inlineStr">
         <is>
-          <t>NOT-READ-41</t>
+          <t>Leads: list renders rows</t>
         </is>
       </c>
       <c r="D129" s="13" t="inlineStr">
@@ -8717,24 +8717,24 @@
       </c>
       <c r="E129" s="10" t="inlineStr">
         <is>
-          <t>GET /notifications -&gt; 200 (loads/lists for authorised user)</t>
+          <t>104 lead rows/links present</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="10" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>WEB-UI</t>
         </is>
       </c>
       <c r="B130" s="10" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="C130" s="10" t="inlineStr">
         <is>
-          <t>NOT-READ-42</t>
+          <t>Web page renders: /leads</t>
         </is>
       </c>
       <c r="D130" s="13" t="inlineStr">
@@ -8744,7 +8744,7 @@
       </c>
       <c r="E130" s="10" t="inlineStr">
         <is>
-          <t>GET /notifications/preferences -&gt; 200 (loads/lists for authorised user)</t>
+          <t>Rendered correctly; saw ["Lead","QA-HVAC"]</t>
         </is>
       </c>
     </row>
@@ -8756,12 +8756,12 @@
       </c>
       <c r="B131" s="10" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Mobile Field App</t>
         </is>
       </c>
       <c r="C131" s="10" t="inlineStr">
         <is>
-          <t>NOT-READ-43</t>
+          <t>MOB-TC-040</t>
         </is>
       </c>
       <c r="D131" s="13" t="inlineStr">
@@ -8771,7 +8771,7 @@
       </c>
       <c r="E131" s="10" t="inlineStr">
         <is>
-          <t>GET /notifications/routing-rules -&gt; 200 (loads/lists for authorised user)</t>
+          <t>Create mobile voice note (contextType=general)</t>
         </is>
       </c>
     </row>
@@ -8783,12 +8783,12 @@
       </c>
       <c r="B132" s="10" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Mobile Field App</t>
         </is>
       </c>
       <c r="C132" s="10" t="inlineStr">
         <is>
-          <t>NOT-RBAC-create_routing_rul</t>
+          <t>MOB-TC-041</t>
         </is>
       </c>
       <c r="D132" s="13" t="inlineStr">
@@ -8798,24 +8798,24 @@
       </c>
       <c r="E132" s="10" t="inlineStr">
         <is>
-          <t>Default-deny on "create routing rule": all 3 unauthorised roles got 403</t>
+          <t>PCI: card number in voice transcript rejected</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="10" t="inlineStr">
         <is>
-          <t>WEB-UI</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B133" s="10" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Mobile Field App</t>
         </is>
       </c>
       <c r="C133" s="10" t="inlineStr">
         <is>
-          <t>Web page renders: /notifications</t>
+          <t>MOB-TC-042</t>
         </is>
       </c>
       <c r="D133" s="13" t="inlineStr">
@@ -8825,24 +8825,24 @@
       </c>
       <c r="E133" s="10" t="inlineStr">
         <is>
-          <t>Rendered correctly; saw ["Notifications"]</t>
+          <t>Voice-note review queue loads</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="10" t="inlineStr">
         <is>
-          <t>WEB-UI</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B134" s="10" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Mobile Field App</t>
         </is>
       </c>
       <c r="C134" s="10" t="inlineStr">
         <is>
-          <t>Web page renders: /settings/notifications/routing</t>
+          <t>MOB-TC-043</t>
         </is>
       </c>
       <c r="D134" s="13" t="inlineStr">
@@ -8852,24 +8852,24 @@
       </c>
       <c r="E134" s="10" t="inlineStr">
         <is>
-          <t>Rendered correctly; saw ["Recipient"]</t>
+          <t>Voice-note list loads</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="10" t="inlineStr">
         <is>
-          <t>WEB-UI</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B135" s="10" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Mobile Field App</t>
         </is>
       </c>
       <c r="C135" s="10" t="inlineStr">
         <is>
-          <t>Web page renders: /settings/notifications</t>
+          <t>MOB-TC-044</t>
         </is>
       </c>
       <c r="D135" s="13" t="inlineStr">
@@ -8879,7 +8879,7 @@
       </c>
       <c r="E135" s="10" t="inlineStr">
         <is>
-          <t>Rendered correctly; saw ["Notification preferences"]</t>
+          <t>Reviewer approves a voice note</t>
         </is>
       </c>
     </row>
@@ -8891,12 +8891,12 @@
       </c>
       <c r="B136" s="10" t="inlineStr">
         <is>
-          <t>Product Management &amp; Catalog</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C136" s="10" t="inlineStr">
         <is>
-          <t>PM-TC-001</t>
+          <t>NOT-TC-001</t>
         </is>
       </c>
       <c r="D136" s="13" t="inlineStr">
@@ -8906,7 +8906,7 @@
       </c>
       <c r="E136" s="10" t="inlineStr">
         <is>
-          <t>Product families 200</t>
+          <t>Notifications inbox list 200</t>
         </is>
       </c>
     </row>
@@ -8918,12 +8918,12 @@
       </c>
       <c r="B137" s="10" t="inlineStr">
         <is>
-          <t>Product Management &amp; Catalog</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C137" s="10" t="inlineStr">
         <is>
-          <t>PM-TC-002</t>
+          <t>NOT-TC-002</t>
         </is>
       </c>
       <c r="D137" s="13" t="inlineStr">
@@ -8933,7 +8933,7 @@
       </c>
       <c r="E137" s="10" t="inlineStr">
         <is>
-          <t>Product categories 200</t>
+          <t>Notifications unread count 200</t>
         </is>
       </c>
     </row>
@@ -8945,12 +8945,12 @@
       </c>
       <c r="B138" s="10" t="inlineStr">
         <is>
-          <t>Product Management &amp; Catalog</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C138" s="10" t="inlineStr">
         <is>
-          <t>PM-TC-003</t>
+          <t>NOT-TC-003</t>
         </is>
       </c>
       <c r="D138" s="13" t="inlineStr">
@@ -8960,7 +8960,7 @@
       </c>
       <c r="E138" s="10" t="inlineStr">
         <is>
-          <t>Product rule sets 200</t>
+          <t>Notifications preferences 200</t>
         </is>
       </c>
     </row>
@@ -8972,12 +8972,12 @@
       </c>
       <c r="B139" s="10" t="inlineStr">
         <is>
-          <t>Product Management &amp; Catalog</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C139" s="10" t="inlineStr">
         <is>
-          <t>PM-TC-004</t>
+          <t>NOT-TC-010</t>
         </is>
       </c>
       <c r="D139" s="13" t="inlineStr">
@@ -8987,7 +8987,7 @@
       </c>
       <c r="E139" s="10" t="inlineStr">
         <is>
-          <t>Product catalog views 200</t>
+          <t>Admin can read routing rules</t>
         </is>
       </c>
     </row>
@@ -8999,12 +8999,12 @@
       </c>
       <c r="B140" s="10" t="inlineStr">
         <is>
-          <t>Product Management &amp; Catalog</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C140" s="10" t="inlineStr">
         <is>
-          <t>PM-TC-010</t>
+          <t>NOT-TC-011</t>
         </is>
       </c>
       <c r="D140" s="13" t="inlineStr">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="E140" s="10" t="inlineStr">
         <is>
-          <t>Create product family</t>
+          <t>Routing rules access for TM controlled (403)</t>
         </is>
       </c>
     </row>
@@ -9026,12 +9026,12 @@
       </c>
       <c r="B141" s="10" t="inlineStr">
         <is>
-          <t>Product Management &amp; Catalog</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C141" s="10" t="inlineStr">
         <is>
-          <t>PM-TC-011</t>
+          <t>NOT-TC-020</t>
         </is>
       </c>
       <c r="D141" s="13" t="inlineStr">
@@ -9041,7 +9041,7 @@
       </c>
       <c r="E141" s="10" t="inlineStr">
         <is>
-          <t>Create product category</t>
+          <t>Mark notifications read</t>
         </is>
       </c>
     </row>
@@ -9053,22 +9053,22 @@
       </c>
       <c r="B142" s="10" t="inlineStr">
         <is>
-          <t>Product Management &amp; Catalog</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C142" s="10" t="inlineStr">
         <is>
-          <t>PM-TC-012</t>
-        </is>
-      </c>
-      <c r="D142" s="13" t="inlineStr">
-        <is>
-          <t>PASS</t>
+          <t>NOT-TC-021</t>
+        </is>
+      </c>
+      <c r="D142" s="14" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="E142" s="10" t="inlineStr">
         <is>
-          <t>SALES_BD_REP denied catalog manage</t>
+          <t>400: A valid notification category is required.</t>
         </is>
       </c>
     </row>
@@ -9080,12 +9080,12 @@
       </c>
       <c r="B143" s="10" t="inlineStr">
         <is>
-          <t>Product Management &amp; Catalog</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C143" s="10" t="inlineStr">
         <is>
-          <t>PM-READ-17</t>
+          <t>NOT-TC-022</t>
         </is>
       </c>
       <c r="D143" s="13" t="inlineStr">
@@ -9095,7 +9095,7 @@
       </c>
       <c r="E143" s="10" t="inlineStr">
         <is>
-          <t>GET /product-management/families -&gt; 200 (loads/lists for authorised user)</t>
+          <t>Create notification routing rule</t>
         </is>
       </c>
     </row>
@@ -9107,12 +9107,12 @@
       </c>
       <c r="B144" s="10" t="inlineStr">
         <is>
-          <t>Product Management &amp; Catalog</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C144" s="10" t="inlineStr">
         <is>
-          <t>PM-READ-18</t>
+          <t>NOT-TC-023</t>
         </is>
       </c>
       <c r="D144" s="13" t="inlineStr">
@@ -9122,7 +9122,7 @@
       </c>
       <c r="E144" s="10" t="inlineStr">
         <is>
-          <t>GET /product-management/categories -&gt; 200 (loads/lists for authorised user)</t>
+          <t>Delete routing rule</t>
         </is>
       </c>
     </row>
@@ -9134,12 +9134,12 @@
       </c>
       <c r="B145" s="10" t="inlineStr">
         <is>
-          <t>Product Management &amp; Catalog</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C145" s="10" t="inlineStr">
         <is>
-          <t>PM-READ-19</t>
+          <t>NOT-TC-024</t>
         </is>
       </c>
       <c r="D145" s="13" t="inlineStr">
@@ -9149,7 +9149,7 @@
       </c>
       <c r="E145" s="10" t="inlineStr">
         <is>
-          <t>GET /product-management/catalog-rule-sets -&gt; 200 (loads/lists for authorised user)</t>
+          <t>TM denied routing-rule creation (admin-gated)</t>
         </is>
       </c>
     </row>
@@ -9161,12 +9161,12 @@
       </c>
       <c r="B146" s="10" t="inlineStr">
         <is>
-          <t>Product Management &amp; Catalog</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C146" s="10" t="inlineStr">
         <is>
-          <t>PM-READ-20</t>
+          <t>NOT-READ-16</t>
         </is>
       </c>
       <c r="D146" s="13" t="inlineStr">
@@ -9176,7 +9176,7 @@
       </c>
       <c r="E146" s="10" t="inlineStr">
         <is>
-          <t>GET /product-management/catalog-views -&gt; 200 (loads/lists for authorised user)</t>
+          <t>GET /notifications/unread-count -&gt; 200 (loads/lists for authorised user)</t>
         </is>
       </c>
     </row>
@@ -9188,12 +9188,12 @@
       </c>
       <c r="B147" s="10" t="inlineStr">
         <is>
-          <t>Product Management &amp; Catalog</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C147" s="10" t="inlineStr">
         <is>
-          <t>PM-READ-21</t>
+          <t>NOT-READ-41</t>
         </is>
       </c>
       <c r="D147" s="13" t="inlineStr">
@@ -9203,7 +9203,7 @@
       </c>
       <c r="E147" s="10" t="inlineStr">
         <is>
-          <t>GET /product-management/catalog-rule-options -&gt; 200 (loads/lists for authorised user)</t>
+          <t>GET /notifications -&gt; 200 (loads/lists for authorised user)</t>
         </is>
       </c>
     </row>
@@ -9215,22 +9215,22 @@
       </c>
       <c r="B148" s="10" t="inlineStr">
         <is>
-          <t>Product Management &amp; Catalog</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C148" s="10" t="inlineStr">
         <is>
-          <t>PM-READ-22</t>
-        </is>
-      </c>
-      <c r="D148" s="14" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+          <t>NOT-READ-42</t>
+        </is>
+      </c>
+      <c r="D148" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="E148" s="10" t="inlineStr">
         <is>
-          <t>GET /product-management/catalog-inclusions -&gt; 405 (needs params or method)</t>
+          <t>GET /notifications/preferences -&gt; 200 (loads/lists for authorised user)</t>
         </is>
       </c>
     </row>
@@ -9242,12 +9242,12 @@
       </c>
       <c r="B149" s="10" t="inlineStr">
         <is>
-          <t>Product Management &amp; Catalog</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C149" s="10" t="inlineStr">
         <is>
-          <t>PM-RBAC-create_product_fam</t>
+          <t>NOT-READ-43</t>
         </is>
       </c>
       <c r="D149" s="13" t="inlineStr">
@@ -9257,24 +9257,24 @@
       </c>
       <c r="E149" s="10" t="inlineStr">
         <is>
-          <t>Default-deny on "create product family": all 4 unauthorised roles got 403</t>
+          <t>GET /notifications/routing-rules -&gt; 200 (loads/lists for authorised user)</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="10" t="inlineStr">
         <is>
-          <t>WEB-UI</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B150" s="10" t="inlineStr">
         <is>
-          <t>Product Management &amp; Catalog</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C150" s="10" t="inlineStr">
         <is>
-          <t>Web page renders: /product-management</t>
+          <t>NOT-RBAC-create_routing_rul</t>
         </is>
       </c>
       <c r="D150" s="13" t="inlineStr">
@@ -9284,24 +9284,24 @@
       </c>
       <c r="E150" s="10" t="inlineStr">
         <is>
-          <t>Rendered correctly; saw ["Product","Pulse"]</t>
+          <t>Default-deny on "create routing rule": all 3 unauthorised roles got 403</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="10" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>WEB-UI</t>
         </is>
       </c>
       <c r="B151" s="10" t="inlineStr">
         <is>
-          <t>Reporting &amp; Dashboards</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C151" s="10" t="inlineStr">
         <is>
-          <t>RPT-TC-001</t>
+          <t>Web page renders: /notifications</t>
         </is>
       </c>
       <c r="D151" s="13" t="inlineStr">
@@ -9311,24 +9311,24 @@
       </c>
       <c r="E151" s="10" t="inlineStr">
         <is>
-          <t>Lead dashboard returns 200 for SUPER_ADMIN</t>
+          <t>Rendered correctly; saw ["Notifications"]</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="10" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>WEB-UI</t>
         </is>
       </c>
       <c r="B152" s="10" t="inlineStr">
         <is>
-          <t>Reporting &amp; Dashboards</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C152" s="10" t="inlineStr">
         <is>
-          <t>RPT-TC-002</t>
+          <t>Web page renders: /settings/notifications/routing</t>
         </is>
       </c>
       <c r="D152" s="13" t="inlineStr">
@@ -9338,24 +9338,24 @@
       </c>
       <c r="E152" s="10" t="inlineStr">
         <is>
-          <t>Training dashboard returns 200 for SUPER_ADMIN</t>
+          <t>Rendered correctly; saw ["Recipient"]</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="10" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>WEB-UI</t>
         </is>
       </c>
       <c r="B153" s="10" t="inlineStr">
         <is>
-          <t>Reporting &amp; Dashboards</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C153" s="10" t="inlineStr">
         <is>
-          <t>RPT-TC-003</t>
+          <t>Web page renders: /settings/notifications</t>
         </is>
       </c>
       <c r="D153" s="13" t="inlineStr">
@@ -9365,7 +9365,7 @@
       </c>
       <c r="E153" s="10" t="inlineStr">
         <is>
-          <t>Executive dashboard returns 200 for SUPER_ADMIN</t>
+          <t>Rendered correctly; saw ["Notification preferences"]</t>
         </is>
       </c>
     </row>
@@ -9377,12 +9377,12 @@
       </c>
       <c r="B154" s="10" t="inlineStr">
         <is>
-          <t>Reporting &amp; Dashboards</t>
+          <t>Product Management &amp; Catalog</t>
         </is>
       </c>
       <c r="C154" s="10" t="inlineStr">
         <is>
-          <t>RPT-TC-020</t>
+          <t>PM-TC-001</t>
         </is>
       </c>
       <c r="D154" s="13" t="inlineStr">
@@ -9392,7 +9392,7 @@
       </c>
       <c r="E154" s="10" t="inlineStr">
         <is>
-          <t>EXECUTIVE can view executive dashboard</t>
+          <t>Product families 200</t>
         </is>
       </c>
     </row>
@@ -9404,12 +9404,12 @@
       </c>
       <c r="B155" s="10" t="inlineStr">
         <is>
-          <t>Reporting &amp; Dashboards</t>
+          <t>Product Management &amp; Catalog</t>
         </is>
       </c>
       <c r="C155" s="10" t="inlineStr">
         <is>
-          <t>RPT-TC-021</t>
+          <t>PM-TC-002</t>
         </is>
       </c>
       <c r="D155" s="13" t="inlineStr">
@@ -9419,7 +9419,7 @@
       </c>
       <c r="E155" s="10" t="inlineStr">
         <is>
-          <t>TM denied executive dashboard (reports.executive gate)</t>
+          <t>Product categories 200</t>
         </is>
       </c>
     </row>
@@ -9431,12 +9431,12 @@
       </c>
       <c r="B156" s="10" t="inlineStr">
         <is>
-          <t>Reporting &amp; Dashboards</t>
+          <t>Product Management &amp; Catalog</t>
         </is>
       </c>
       <c r="C156" s="10" t="inlineStr">
         <is>
-          <t>RPT-TC-039</t>
+          <t>PM-TC-003</t>
         </is>
       </c>
       <c r="D156" s="13" t="inlineStr">
@@ -9446,7 +9446,7 @@
       </c>
       <c r="E156" s="10" t="inlineStr">
         <is>
-          <t>Stale/neglected accounts report 200</t>
+          <t>Product rule sets 200</t>
         </is>
       </c>
     </row>
@@ -9458,12 +9458,12 @@
       </c>
       <c r="B157" s="10" t="inlineStr">
         <is>
-          <t>Reporting &amp; Dashboards</t>
+          <t>Product Management &amp; Catalog</t>
         </is>
       </c>
       <c r="C157" s="10" t="inlineStr">
         <is>
-          <t>RPT-TC-003b</t>
+          <t>PM-TC-004</t>
         </is>
       </c>
       <c r="D157" s="13" t="inlineStr">
@@ -9473,7 +9473,7 @@
       </c>
       <c r="E157" s="10" t="inlineStr">
         <is>
-          <t>Threshold settings readable</t>
+          <t>Product catalog views 200</t>
         </is>
       </c>
     </row>
@@ -9485,12 +9485,12 @@
       </c>
       <c r="B158" s="10" t="inlineStr">
         <is>
-          <t>Reporting &amp; Dashboards</t>
+          <t>Product Management &amp; Catalog</t>
         </is>
       </c>
       <c r="C158" s="10" t="inlineStr">
         <is>
-          <t>RPT-TC-022b</t>
+          <t>PM-TC-010</t>
         </is>
       </c>
       <c r="D158" s="13" t="inlineStr">
@@ -9500,7 +9500,7 @@
       </c>
       <c r="E158" s="10" t="inlineStr">
         <is>
-          <t>TM threshold-settings access controlled (200)</t>
+          <t>Create product family</t>
         </is>
       </c>
     </row>
@@ -9512,12 +9512,12 @@
       </c>
       <c r="B159" s="10" t="inlineStr">
         <is>
-          <t>Reporting &amp; Dashboards</t>
+          <t>Product Management &amp; Catalog</t>
         </is>
       </c>
       <c r="C159" s="10" t="inlineStr">
         <is>
-          <t>RPT-TC-064</t>
+          <t>PM-TC-011</t>
         </is>
       </c>
       <c r="D159" s="13" t="inlineStr">
@@ -9527,7 +9527,7 @@
       </c>
       <c r="E159" s="10" t="inlineStr">
         <is>
-          <t>List report definitions</t>
+          <t>Create product category</t>
         </is>
       </c>
     </row>
@@ -9539,12 +9539,12 @@
       </c>
       <c r="B160" s="10" t="inlineStr">
         <is>
-          <t>Reporting &amp; Dashboards</t>
+          <t>Product Management &amp; Catalog</t>
         </is>
       </c>
       <c r="C160" s="10" t="inlineStr">
         <is>
-          <t>RPT-RUN-lead_funnel</t>
+          <t>PM-TC-012</t>
         </is>
       </c>
       <c r="D160" s="13" t="inlineStr">
@@ -9554,7 +9554,7 @@
       </c>
       <c r="E160" s="10" t="inlineStr">
         <is>
-          <t>Run ad-hoc report lead_funnel</t>
+          <t>SALES_BD_REP denied catalog manage</t>
         </is>
       </c>
     </row>
@@ -9566,12 +9566,12 @@
       </c>
       <c r="B161" s="10" t="inlineStr">
         <is>
-          <t>Reporting &amp; Dashboards</t>
+          <t>Product Management &amp; Catalog</t>
         </is>
       </c>
       <c r="C161" s="10" t="inlineStr">
         <is>
-          <t>RPT-RUN-training_compliance</t>
+          <t>PM-READ-17</t>
         </is>
       </c>
       <c r="D161" s="13" t="inlineStr">
@@ -9581,7 +9581,7 @@
       </c>
       <c r="E161" s="10" t="inlineStr">
         <is>
-          <t>Run ad-hoc report training_compliance</t>
+          <t>GET /product-management/families -&gt; 200 (loads/lists for authorised user)</t>
         </is>
       </c>
     </row>
@@ -9593,12 +9593,12 @@
       </c>
       <c r="B162" s="10" t="inlineStr">
         <is>
-          <t>Reporting &amp; Dashboards</t>
+          <t>Product Management &amp; Catalog</t>
         </is>
       </c>
       <c r="C162" s="10" t="inlineStr">
         <is>
-          <t>RPT-RUN-consignment_audit_status</t>
+          <t>PM-READ-18</t>
         </is>
       </c>
       <c r="D162" s="13" t="inlineStr">
@@ -9608,7 +9608,7 @@
       </c>
       <c r="E162" s="10" t="inlineStr">
         <is>
-          <t>Run ad-hoc report consignment_audit_status</t>
+          <t>GET /product-management/categories -&gt; 200 (loads/lists for authorised user)</t>
         </is>
       </c>
     </row>
@@ -9620,12 +9620,12 @@
       </c>
       <c r="B163" s="10" t="inlineStr">
         <is>
-          <t>Reporting &amp; Dashboards</t>
+          <t>Product Management &amp; Catalog</t>
         </is>
       </c>
       <c r="C163" s="10" t="inlineStr">
         <is>
-          <t>RPT-RUN-field_activity</t>
+          <t>PM-READ-19</t>
         </is>
       </c>
       <c r="D163" s="13" t="inlineStr">
@@ -9635,7 +9635,7 @@
       </c>
       <c r="E163" s="10" t="inlineStr">
         <is>
-          <t>Run ad-hoc report field_activity</t>
+          <t>GET /product-management/catalog-rule-sets -&gt; 200 (loads/lists for authorised user)</t>
         </is>
       </c>
     </row>
@@ -9647,12 +9647,12 @@
       </c>
       <c r="B164" s="10" t="inlineStr">
         <is>
-          <t>Reporting &amp; Dashboards</t>
+          <t>Product Management &amp; Catalog</t>
         </is>
       </c>
       <c r="C164" s="10" t="inlineStr">
         <is>
-          <t>RPT-READ-13</t>
+          <t>PM-READ-20</t>
         </is>
       </c>
       <c r="D164" s="13" t="inlineStr">
@@ -9662,7 +9662,7 @@
       </c>
       <c r="E164" s="10" t="inlineStr">
         <is>
-          <t>GET /reports/definitions -&gt; 200 (loads/lists for authorised user)</t>
+          <t>GET /product-management/catalog-views -&gt; 200 (loads/lists for authorised user)</t>
         </is>
       </c>
     </row>
@@ -9674,12 +9674,12 @@
       </c>
       <c r="B165" s="10" t="inlineStr">
         <is>
-          <t>Reporting &amp; Dashboards</t>
+          <t>Product Management &amp; Catalog</t>
         </is>
       </c>
       <c r="C165" s="10" t="inlineStr">
         <is>
-          <t>RPT-READ-14</t>
+          <t>PM-READ-21</t>
         </is>
       </c>
       <c r="D165" s="13" t="inlineStr">
@@ -9689,7 +9689,7 @@
       </c>
       <c r="E165" s="10" t="inlineStr">
         <is>
-          <t>GET /reports/stale-accounts -&gt; 200 (loads/lists for authorised user)</t>
+          <t>GET /product-management/catalog-rule-options -&gt; 200 (loads/lists for authorised user)</t>
         </is>
       </c>
     </row>
@@ -9701,22 +9701,22 @@
       </c>
       <c r="B166" s="10" t="inlineStr">
         <is>
-          <t>Reporting &amp; Dashboards</t>
+          <t>Product Management &amp; Catalog</t>
         </is>
       </c>
       <c r="C166" s="10" t="inlineStr">
         <is>
-          <t>RPT-READ-15</t>
-        </is>
-      </c>
-      <c r="D166" s="13" t="inlineStr">
-        <is>
-          <t>PASS</t>
+          <t>PM-READ-22</t>
+        </is>
+      </c>
+      <c r="D166" s="14" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="E166" s="10" t="inlineStr">
         <is>
-          <t>GET /reports/threshold-settings -&gt; 200 (loads/lists for authorised user)</t>
+          <t>GET /product-management/catalog-inclusions -&gt; 405 (needs params or method)</t>
         </is>
       </c>
     </row>
@@ -9728,12 +9728,12 @@
       </c>
       <c r="B167" s="10" t="inlineStr">
         <is>
-          <t>Reporting &amp; Dashboards</t>
+          <t>Product Management &amp; Catalog</t>
         </is>
       </c>
       <c r="C167" s="10" t="inlineStr">
         <is>
-          <t>RPT-RBAC-executive_dashboar</t>
+          <t>PM-RBAC-create_product_fam</t>
         </is>
       </c>
       <c r="D167" s="13" t="inlineStr">
@@ -9743,7 +9743,7 @@
       </c>
       <c r="E167" s="10" t="inlineStr">
         <is>
-          <t>Default-deny on "executive dashboard": all 4 unauthorised roles got 403</t>
+          <t>Default-deny on "create product family": all 4 unauthorised roles got 403</t>
         </is>
       </c>
     </row>
@@ -9755,12 +9755,12 @@
       </c>
       <c r="B168" s="10" t="inlineStr">
         <is>
-          <t>Reporting &amp; Dashboards</t>
+          <t>Product Management &amp; Catalog</t>
         </is>
       </c>
       <c r="C168" s="10" t="inlineStr">
         <is>
-          <t>Reports: dashboard Export control present (CSV/Excel/PDF)</t>
+          <t>Web page renders: /product-management</t>
         </is>
       </c>
       <c r="D168" s="13" t="inlineStr">
@@ -9770,14 +9770,14 @@
       </c>
       <c r="E168" s="10" t="inlineStr">
         <is>
-          <t>Export button rendered on dashboard</t>
+          <t>Rendered correctly; saw ["Product","Pulse"]</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="10" t="inlineStr">
         <is>
-          <t>WEB-UI</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B169" s="10" t="inlineStr">
@@ -9787,7 +9787,7 @@
       </c>
       <c r="C169" s="10" t="inlineStr">
         <is>
-          <t>Web page renders: /reports</t>
+          <t>RPT-TC-001</t>
         </is>
       </c>
       <c r="D169" s="13" t="inlineStr">
@@ -9797,7 +9797,7 @@
       </c>
       <c r="E169" s="10" t="inlineStr">
         <is>
-          <t>Rendered correctly; saw ["Reports","Export"]</t>
+          <t>Lead dashboard returns 200 for SUPER_ADMIN</t>
         </is>
       </c>
     </row>
@@ -9809,12 +9809,12 @@
       </c>
       <c r="B170" s="10" t="inlineStr">
         <is>
-          <t>Territory</t>
+          <t>Reporting &amp; Dashboards</t>
         </is>
       </c>
       <c r="C170" s="10" t="inlineStr">
         <is>
-          <t>TER-TC-001</t>
+          <t>RPT-TC-002</t>
         </is>
       </c>
       <c r="D170" s="13" t="inlineStr">
@@ -9824,7 +9824,7 @@
       </c>
       <c r="E170" s="10" t="inlineStr">
         <is>
-          <t>Territory list 200</t>
+          <t>Training dashboard returns 200 for SUPER_ADMIN</t>
         </is>
       </c>
     </row>
@@ -9836,12 +9836,12 @@
       </c>
       <c r="B171" s="10" t="inlineStr">
         <is>
-          <t>Territory</t>
+          <t>Reporting &amp; Dashboards</t>
         </is>
       </c>
       <c r="C171" s="10" t="inlineStr">
         <is>
-          <t>TER-TC-002</t>
+          <t>RPT-TC-003</t>
         </is>
       </c>
       <c r="D171" s="13" t="inlineStr">
@@ -9851,7 +9851,7 @@
       </c>
       <c r="E171" s="10" t="inlineStr">
         <is>
-          <t>Territory regions 200</t>
+          <t>Executive dashboard returns 200 for SUPER_ADMIN</t>
         </is>
       </c>
     </row>
@@ -9863,12 +9863,12 @@
       </c>
       <c r="B172" s="10" t="inlineStr">
         <is>
-          <t>Territory</t>
+          <t>Reporting &amp; Dashboards</t>
         </is>
       </c>
       <c r="C172" s="10" t="inlineStr">
         <is>
-          <t>TER-TC-003</t>
+          <t>RPT-TC-020</t>
         </is>
       </c>
       <c r="D172" s="13" t="inlineStr">
@@ -9878,7 +9878,7 @@
       </c>
       <c r="E172" s="10" t="inlineStr">
         <is>
-          <t>Territory map 200</t>
+          <t>EXECUTIVE can view executive dashboard</t>
         </is>
       </c>
     </row>
@@ -9890,12 +9890,12 @@
       </c>
       <c r="B173" s="10" t="inlineStr">
         <is>
-          <t>Territory</t>
+          <t>Reporting &amp; Dashboards</t>
         </is>
       </c>
       <c r="C173" s="10" t="inlineStr">
         <is>
-          <t>TER-TC-004</t>
+          <t>RPT-TC-021</t>
         </is>
       </c>
       <c r="D173" s="13" t="inlineStr">
@@ -9905,7 +9905,7 @@
       </c>
       <c r="E173" s="10" t="inlineStr">
         <is>
-          <t>Territory dashboard 200</t>
+          <t>TM denied executive dashboard (reports.executive gate)</t>
         </is>
       </c>
     </row>
@@ -9917,12 +9917,12 @@
       </c>
       <c r="B174" s="10" t="inlineStr">
         <is>
-          <t>Territory</t>
+          <t>Reporting &amp; Dashboards</t>
         </is>
       </c>
       <c r="C174" s="10" t="inlineStr">
         <is>
-          <t>TER-TC-010</t>
+          <t>RPT-TC-039</t>
         </is>
       </c>
       <c r="D174" s="13" t="inlineStr">
@@ -9932,7 +9932,7 @@
       </c>
       <c r="E174" s="10" t="inlineStr">
         <is>
-          <t>TM can read territories</t>
+          <t>Stale/neglected accounts report 200</t>
         </is>
       </c>
     </row>
@@ -9944,12 +9944,12 @@
       </c>
       <c r="B175" s="10" t="inlineStr">
         <is>
-          <t>Territory</t>
+          <t>Reporting &amp; Dashboards</t>
         </is>
       </c>
       <c r="C175" s="10" t="inlineStr">
         <is>
-          <t>TER-TC-020</t>
+          <t>RPT-TC-003b</t>
         </is>
       </c>
       <c r="D175" s="13" t="inlineStr">
@@ -9959,7 +9959,7 @@
       </c>
       <c r="E175" s="10" t="inlineStr">
         <is>
-          <t>Territory assignable users</t>
+          <t>Threshold settings readable</t>
         </is>
       </c>
     </row>
@@ -9971,12 +9971,12 @@
       </c>
       <c r="B176" s="10" t="inlineStr">
         <is>
-          <t>Territory</t>
+          <t>Reporting &amp; Dashboards</t>
         </is>
       </c>
       <c r="C176" s="10" t="inlineStr">
         <is>
-          <t>TER-TC-021</t>
+          <t>RPT-TC-022b</t>
         </is>
       </c>
       <c r="D176" s="13" t="inlineStr">
@@ -9986,7 +9986,7 @@
       </c>
       <c r="E176" s="10" t="inlineStr">
         <is>
-          <t>Territory policy</t>
+          <t>TM threshold-settings access controlled (200)</t>
         </is>
       </c>
     </row>
@@ -9998,12 +9998,12 @@
       </c>
       <c r="B177" s="10" t="inlineStr">
         <is>
-          <t>Territory</t>
+          <t>Reporting &amp; Dashboards</t>
         </is>
       </c>
       <c r="C177" s="10" t="inlineStr">
         <is>
-          <t>TER-TC-023</t>
+          <t>RPT-TC-064</t>
         </is>
       </c>
       <c r="D177" s="13" t="inlineStr">
@@ -10013,7 +10013,7 @@
       </c>
       <c r="E177" s="10" t="inlineStr">
         <is>
-          <t>Territory shipping centers</t>
+          <t>List report definitions</t>
         </is>
       </c>
     </row>
@@ -10025,12 +10025,12 @@
       </c>
       <c r="B178" s="10" t="inlineStr">
         <is>
-          <t>Territory</t>
+          <t>Reporting &amp; Dashboards</t>
         </is>
       </c>
       <c r="C178" s="10" t="inlineStr">
         <is>
-          <t>TER-READ-01</t>
+          <t>RPT-RUN-lead_funnel</t>
         </is>
       </c>
       <c r="D178" s="13" t="inlineStr">
@@ -10040,7 +10040,7 @@
       </c>
       <c r="E178" s="10" t="inlineStr">
         <is>
-          <t>GET /territories/regions -&gt; 200 (loads/lists for authorised user)</t>
+          <t>Run ad-hoc report lead_funnel</t>
         </is>
       </c>
     </row>
@@ -10052,12 +10052,12 @@
       </c>
       <c r="B179" s="10" t="inlineStr">
         <is>
-          <t>Territory</t>
+          <t>Reporting &amp; Dashboards</t>
         </is>
       </c>
       <c r="C179" s="10" t="inlineStr">
         <is>
-          <t>TER-READ-02</t>
+          <t>RPT-RUN-training_compliance</t>
         </is>
       </c>
       <c r="D179" s="13" t="inlineStr">
@@ -10067,7 +10067,7 @@
       </c>
       <c r="E179" s="10" t="inlineStr">
         <is>
-          <t>GET /territories/map -&gt; 200 (loads/lists for authorised user)</t>
+          <t>Run ad-hoc report training_compliance</t>
         </is>
       </c>
     </row>
@@ -10079,12 +10079,12 @@
       </c>
       <c r="B180" s="10" t="inlineStr">
         <is>
-          <t>Territory</t>
+          <t>Reporting &amp; Dashboards</t>
         </is>
       </c>
       <c r="C180" s="10" t="inlineStr">
         <is>
-          <t>TER-READ-03</t>
+          <t>RPT-RUN-consignment_audit_status</t>
         </is>
       </c>
       <c r="D180" s="13" t="inlineStr">
@@ -10094,7 +10094,7 @@
       </c>
       <c r="E180" s="10" t="inlineStr">
         <is>
-          <t>GET /territories/dashboard -&gt; 200 (loads/lists for authorised user)</t>
+          <t>Run ad-hoc report consignment_audit_status</t>
         </is>
       </c>
     </row>
@@ -10106,12 +10106,12 @@
       </c>
       <c r="B181" s="10" t="inlineStr">
         <is>
-          <t>Territory</t>
+          <t>Reporting &amp; Dashboards</t>
         </is>
       </c>
       <c r="C181" s="10" t="inlineStr">
         <is>
-          <t>TER-READ-38</t>
+          <t>RPT-RUN-field_activity</t>
         </is>
       </c>
       <c r="D181" s="13" t="inlineStr">
@@ -10121,24 +10121,24 @@
       </c>
       <c r="E181" s="10" t="inlineStr">
         <is>
-          <t>GET /territories -&gt; 200 (loads/lists for authorised user)</t>
+          <t>Run ad-hoc report field_activity</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="10" t="inlineStr">
         <is>
-          <t>WEB-UI</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B182" s="10" t="inlineStr">
         <is>
-          <t>Territory</t>
+          <t>Reporting &amp; Dashboards</t>
         </is>
       </c>
       <c r="C182" s="10" t="inlineStr">
         <is>
-          <t>Web page renders: /territories</t>
+          <t>RPT-READ-13</t>
         </is>
       </c>
       <c r="D182" s="13" t="inlineStr">
@@ -10148,24 +10148,24 @@
       </c>
       <c r="E182" s="10" t="inlineStr">
         <is>
-          <t>Rendered correctly; saw ["Territor","Pulse"]</t>
+          <t>GET /reports/definitions -&gt; 200 (loads/lists for authorised user)</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="10" t="inlineStr">
         <is>
-          <t>WEB-UI</t>
+          <t>API</t>
         </is>
       </c>
       <c r="B183" s="10" t="inlineStr">
         <is>
-          <t>Territory</t>
+          <t>Reporting &amp; Dashboards</t>
         </is>
       </c>
       <c r="C183" s="10" t="inlineStr">
         <is>
-          <t>Web page renders: /territory_map</t>
+          <t>RPT-READ-14</t>
         </is>
       </c>
       <c r="D183" s="13" t="inlineStr">
@@ -10175,7 +10175,7 @@
       </c>
       <c r="E183" s="10" t="inlineStr">
         <is>
-          <t>Rendered correctly; saw ["Pulse"]</t>
+          <t>GET /reports/stale-accounts -&gt; 200 (loads/lists for authorised user)</t>
         </is>
       </c>
     </row>
@@ -10187,12 +10187,12 @@
       </c>
       <c r="B184" s="10" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Reporting &amp; Dashboards</t>
         </is>
       </c>
       <c r="C184" s="10" t="inlineStr">
         <is>
-          <t>TRN-TC-001</t>
+          <t>RPT-READ-15</t>
         </is>
       </c>
       <c r="D184" s="13" t="inlineStr">
@@ -10202,7 +10202,7 @@
       </c>
       <c r="E184" s="10" t="inlineStr">
         <is>
-          <t>Training sessions 200</t>
+          <t>GET /reports/threshold-settings -&gt; 200 (loads/lists for authorised user)</t>
         </is>
       </c>
     </row>
@@ -10214,12 +10214,12 @@
       </c>
       <c r="B185" s="10" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Reporting &amp; Dashboards</t>
         </is>
       </c>
       <c r="C185" s="10" t="inlineStr">
         <is>
-          <t>TRN-TC-002</t>
+          <t>RPT-RBAC-executive_dashboar</t>
         </is>
       </c>
       <c r="D185" s="13" t="inlineStr">
@@ -10229,24 +10229,24 @@
       </c>
       <c r="E185" s="10" t="inlineStr">
         <is>
-          <t>Training overview 200</t>
+          <t>Default-deny on "executive dashboard": all 4 unauthorised roles got 403</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="10" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>WEB-UI</t>
         </is>
       </c>
       <c r="B186" s="10" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Reporting &amp; Dashboards</t>
         </is>
       </c>
       <c r="C186" s="10" t="inlineStr">
         <is>
-          <t>TRN-TC-003</t>
+          <t>Reports: dashboard Export control present (CSV/Excel/PDF)</t>
         </is>
       </c>
       <c r="D186" s="13" t="inlineStr">
@@ -10256,24 +10256,24 @@
       </c>
       <c r="E186" s="10" t="inlineStr">
         <is>
-          <t>Training catalog 200</t>
+          <t>Export button rendered on dashboard</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="10" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>WEB-UI</t>
         </is>
       </c>
       <c r="B187" s="10" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Reporting &amp; Dashboards</t>
         </is>
       </c>
       <c r="C187" s="10" t="inlineStr">
         <is>
-          <t>TRN-TC-004</t>
+          <t>Web page renders: /reports</t>
         </is>
       </c>
       <c r="D187" s="13" t="inlineStr">
@@ -10283,7 +10283,7 @@
       </c>
       <c r="E187" s="10" t="inlineStr">
         <is>
-          <t>Training trainers 200</t>
+          <t>Rendered correctly; saw ["Reports","Export"]</t>
         </is>
       </c>
     </row>
@@ -10295,12 +10295,12 @@
       </c>
       <c r="B188" s="10" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Territory</t>
         </is>
       </c>
       <c r="C188" s="10" t="inlineStr">
         <is>
-          <t>TRN-TC-010</t>
+          <t>TER-TC-001</t>
         </is>
       </c>
       <c r="D188" s="13" t="inlineStr">
@@ -10310,7 +10310,7 @@
       </c>
       <c r="E188" s="10" t="inlineStr">
         <is>
-          <t>TRAINING_OPS can read sessions</t>
+          <t>Territory list 200</t>
         </is>
       </c>
     </row>
@@ -10322,22 +10322,22 @@
       </c>
       <c r="B189" s="10" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Territory</t>
         </is>
       </c>
       <c r="C189" s="10" t="inlineStr">
         <is>
-          <t>TRN-TC-020</t>
-        </is>
-      </c>
-      <c r="D189" s="14" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+          <t>TER-TC-002</t>
+        </is>
+      </c>
+      <c r="D189" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="E189" s="10" t="inlineStr">
         <is>
-          <t>schedule session -&gt; 400: Training type not found</t>
+          <t>Territory regions 200</t>
         </is>
       </c>
     </row>
@@ -10349,12 +10349,12 @@
       </c>
       <c r="B190" s="10" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Territory</t>
         </is>
       </c>
       <c r="C190" s="10" t="inlineStr">
         <is>
-          <t>TRN-TC-023</t>
+          <t>TER-TC-003</t>
         </is>
       </c>
       <c r="D190" s="13" t="inlineStr">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="E190" s="10" t="inlineStr">
         <is>
-          <t>FINANCE denied training.schedule</t>
+          <t>Territory map 200</t>
         </is>
       </c>
     </row>
@@ -10376,12 +10376,12 @@
       </c>
       <c r="B191" s="10" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Territory</t>
         </is>
       </c>
       <c r="C191" s="10" t="inlineStr">
         <is>
-          <t>TRN-READ-04</t>
+          <t>TER-TC-004</t>
         </is>
       </c>
       <c r="D191" s="13" t="inlineStr">
@@ -10391,7 +10391,7 @@
       </c>
       <c r="E191" s="10" t="inlineStr">
         <is>
-          <t>GET /training/overview -&gt; 200 (loads/lists for authorised user)</t>
+          <t>Territory dashboard 200</t>
         </is>
       </c>
     </row>
@@ -10403,12 +10403,12 @@
       </c>
       <c r="B192" s="10" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Territory</t>
         </is>
       </c>
       <c r="C192" s="10" t="inlineStr">
         <is>
-          <t>TRN-READ-05</t>
+          <t>TER-TC-010</t>
         </is>
       </c>
       <c r="D192" s="13" t="inlineStr">
@@ -10418,7 +10418,7 @@
       </c>
       <c r="E192" s="10" t="inlineStr">
         <is>
-          <t>GET /training/recertification -&gt; 200 (loads/lists for authorised user)</t>
+          <t>TM can read territories</t>
         </is>
       </c>
     </row>
@@ -10430,12 +10430,12 @@
       </c>
       <c r="B193" s="10" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Territory</t>
         </is>
       </c>
       <c r="C193" s="10" t="inlineStr">
         <is>
-          <t>TRN-READ-06</t>
+          <t>TER-TC-020</t>
         </is>
       </c>
       <c r="D193" s="13" t="inlineStr">
@@ -10445,7 +10445,7 @@
       </c>
       <c r="E193" s="10" t="inlineStr">
         <is>
-          <t>GET /training/coaching -&gt; 200 (loads/lists for authorised user)</t>
+          <t>Territory assignable users</t>
         </is>
       </c>
     </row>
@@ -10457,12 +10457,12 @@
       </c>
       <c r="B194" s="10" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Territory</t>
         </is>
       </c>
       <c r="C194" s="10" t="inlineStr">
         <is>
-          <t>TRN-READ-07</t>
+          <t>TER-TC-021</t>
         </is>
       </c>
       <c r="D194" s="13" t="inlineStr">
@@ -10472,7 +10472,7 @@
       </c>
       <c r="E194" s="10" t="inlineStr">
         <is>
-          <t>GET /training/territory-penetration -&gt; 200 (loads/lists for authorised user)</t>
+          <t>Territory policy</t>
         </is>
       </c>
     </row>
@@ -10484,12 +10484,12 @@
       </c>
       <c r="B195" s="10" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Territory</t>
         </is>
       </c>
       <c r="C195" s="10" t="inlineStr">
         <is>
-          <t>TRN-READ-08</t>
+          <t>TER-TC-023</t>
         </is>
       </c>
       <c r="D195" s="13" t="inlineStr">
@@ -10499,7 +10499,7 @@
       </c>
       <c r="E195" s="10" t="inlineStr">
         <is>
-          <t>GET /training/accounts -&gt; 200 (loads/lists for authorised user)</t>
+          <t>Territory shipping centers</t>
         </is>
       </c>
     </row>
@@ -10511,12 +10511,12 @@
       </c>
       <c r="B196" s="10" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Territory</t>
         </is>
       </c>
       <c r="C196" s="10" t="inlineStr">
         <is>
-          <t>TRN-READ-09</t>
+          <t>TER-READ-01</t>
         </is>
       </c>
       <c r="D196" s="13" t="inlineStr">
@@ -10526,7 +10526,7 @@
       </c>
       <c r="E196" s="10" t="inlineStr">
         <is>
-          <t>GET /training/ops -&gt; 200 (loads/lists for authorised user)</t>
+          <t>GET /territories/regions -&gt; 200 (loads/lists for authorised user)</t>
         </is>
       </c>
     </row>
@@ -10538,12 +10538,12 @@
       </c>
       <c r="B197" s="10" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Territory</t>
         </is>
       </c>
       <c r="C197" s="10" t="inlineStr">
         <is>
-          <t>TRN-READ-10</t>
+          <t>TER-READ-02</t>
         </is>
       </c>
       <c r="D197" s="13" t="inlineStr">
@@ -10553,7 +10553,7 @@
       </c>
       <c r="E197" s="10" t="inlineStr">
         <is>
-          <t>GET /training/reporting -&gt; 200 (loads/lists for authorised user)</t>
+          <t>GET /territories/map -&gt; 200 (loads/lists for authorised user)</t>
         </is>
       </c>
     </row>
@@ -10565,12 +10565,12 @@
       </c>
       <c r="B198" s="10" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Territory</t>
         </is>
       </c>
       <c r="C198" s="10" t="inlineStr">
         <is>
-          <t>TRN-READ-39</t>
+          <t>TER-READ-03</t>
         </is>
       </c>
       <c r="D198" s="13" t="inlineStr">
@@ -10580,39 +10580,525 @@
       </c>
       <c r="E198" s="10" t="inlineStr">
         <is>
-          <t>GET /training/sessions -&gt; 200 (loads/lists for authorised user)</t>
+          <t>GET /territories/dashboard -&gt; 200 (loads/lists for authorised user)</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="10" t="inlineStr">
         <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B199" s="10" t="inlineStr">
+        <is>
+          <t>Territory</t>
+        </is>
+      </c>
+      <c r="C199" s="10" t="inlineStr">
+        <is>
+          <t>TER-READ-38</t>
+        </is>
+      </c>
+      <c r="D199" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E199" s="10" t="inlineStr">
+        <is>
+          <t>GET /territories -&gt; 200 (loads/lists for authorised user)</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="10" t="inlineStr">
+        <is>
           <t>WEB-UI</t>
         </is>
       </c>
-      <c r="B199" s="10" t="inlineStr">
+      <c r="B200" s="10" t="inlineStr">
+        <is>
+          <t>Territory</t>
+        </is>
+      </c>
+      <c r="C200" s="10" t="inlineStr">
+        <is>
+          <t>Web page renders: /territories</t>
+        </is>
+      </c>
+      <c r="D200" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E200" s="10" t="inlineStr">
+        <is>
+          <t>Rendered correctly; saw ["Territor","Pulse"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="10" t="inlineStr">
+        <is>
+          <t>WEB-UI</t>
+        </is>
+      </c>
+      <c r="B201" s="10" t="inlineStr">
+        <is>
+          <t>Territory</t>
+        </is>
+      </c>
+      <c r="C201" s="10" t="inlineStr">
+        <is>
+          <t>Web page renders: /territory_map</t>
+        </is>
+      </c>
+      <c r="D201" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E201" s="10" t="inlineStr">
+        <is>
+          <t>Rendered correctly; saw ["Pulse"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B202" s="10" t="inlineStr">
         <is>
           <t>Training</t>
         </is>
       </c>
-      <c r="C199" s="10" t="inlineStr">
+      <c r="C202" s="10" t="inlineStr">
+        <is>
+          <t>TRN-TC-001</t>
+        </is>
+      </c>
+      <c r="D202" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E202" s="10" t="inlineStr">
+        <is>
+          <t>Training sessions 200</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B203" s="10" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="C203" s="10" t="inlineStr">
+        <is>
+          <t>TRN-TC-002</t>
+        </is>
+      </c>
+      <c r="D203" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E203" s="10" t="inlineStr">
+        <is>
+          <t>Training overview 200</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B204" s="10" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="C204" s="10" t="inlineStr">
+        <is>
+          <t>TRN-TC-003</t>
+        </is>
+      </c>
+      <c r="D204" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E204" s="10" t="inlineStr">
+        <is>
+          <t>Training catalog 200</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B205" s="10" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="C205" s="10" t="inlineStr">
+        <is>
+          <t>TRN-TC-004</t>
+        </is>
+      </c>
+      <c r="D205" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E205" s="10" t="inlineStr">
+        <is>
+          <t>Training trainers 200</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B206" s="10" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="C206" s="10" t="inlineStr">
+        <is>
+          <t>TRN-TC-010</t>
+        </is>
+      </c>
+      <c r="D206" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E206" s="10" t="inlineStr">
+        <is>
+          <t>TRAINING_OPS can read sessions</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B207" s="10" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="C207" s="10" t="inlineStr">
+        <is>
+          <t>TRN-TC-020</t>
+        </is>
+      </c>
+      <c r="D207" s="14" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="E207" s="10" t="inlineStr">
+        <is>
+          <t>schedule session -&gt; 400: Training type not found</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B208" s="10" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="C208" s="10" t="inlineStr">
+        <is>
+          <t>TRN-TC-023</t>
+        </is>
+      </c>
+      <c r="D208" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E208" s="10" t="inlineStr">
+        <is>
+          <t>FINANCE denied training.schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B209" s="10" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="C209" s="10" t="inlineStr">
+        <is>
+          <t>TRN-READ-04</t>
+        </is>
+      </c>
+      <c r="D209" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E209" s="10" t="inlineStr">
+        <is>
+          <t>GET /training/overview -&gt; 200 (loads/lists for authorised user)</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B210" s="10" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="C210" s="10" t="inlineStr">
+        <is>
+          <t>TRN-READ-05</t>
+        </is>
+      </c>
+      <c r="D210" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E210" s="10" t="inlineStr">
+        <is>
+          <t>GET /training/recertification -&gt; 200 (loads/lists for authorised user)</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B211" s="10" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="C211" s="10" t="inlineStr">
+        <is>
+          <t>TRN-READ-06</t>
+        </is>
+      </c>
+      <c r="D211" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E211" s="10" t="inlineStr">
+        <is>
+          <t>GET /training/coaching -&gt; 200 (loads/lists for authorised user)</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B212" s="10" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="C212" s="10" t="inlineStr">
+        <is>
+          <t>TRN-READ-07</t>
+        </is>
+      </c>
+      <c r="D212" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E212" s="10" t="inlineStr">
+        <is>
+          <t>GET /training/territory-penetration -&gt; 200 (loads/lists for authorised user)</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B213" s="10" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="C213" s="10" t="inlineStr">
+        <is>
+          <t>TRN-READ-08</t>
+        </is>
+      </c>
+      <c r="D213" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E213" s="10" t="inlineStr">
+        <is>
+          <t>GET /training/accounts -&gt; 200 (loads/lists for authorised user)</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B214" s="10" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="C214" s="10" t="inlineStr">
+        <is>
+          <t>TRN-READ-09</t>
+        </is>
+      </c>
+      <c r="D214" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E214" s="10" t="inlineStr">
+        <is>
+          <t>GET /training/ops -&gt; 200 (loads/lists for authorised user)</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B215" s="10" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="C215" s="10" t="inlineStr">
+        <is>
+          <t>TRN-READ-10</t>
+        </is>
+      </c>
+      <c r="D215" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E215" s="10" t="inlineStr">
+        <is>
+          <t>GET /training/reporting -&gt; 200 (loads/lists for authorised user)</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="10" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="B216" s="10" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="C216" s="10" t="inlineStr">
+        <is>
+          <t>TRN-READ-39</t>
+        </is>
+      </c>
+      <c r="D216" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E216" s="10" t="inlineStr">
+        <is>
+          <t>GET /training/sessions -&gt; 200 (loads/lists for authorised user)</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="10" t="inlineStr">
+        <is>
+          <t>WEB-UI</t>
+        </is>
+      </c>
+      <c r="B217" s="10" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="C217" s="10" t="inlineStr">
         <is>
           <t>Web page renders: /training</t>
         </is>
       </c>
-      <c r="D199" s="13" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="E199" s="10" t="inlineStr">
+      <c r="D217" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E217" s="10" t="inlineStr">
         <is>
           <t>Rendered correctly; saw ["Training","Pulse"]</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:E199"/>
+  <autoFilter ref="A3:E217"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>